<commit_message>
Updated excluded variable text.
</commit_message>
<xml_diff>
--- a/assets_output/09_logistic_regression_blocks.xlsx
+++ b/assets_output/09_logistic_regression_blocks.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="156">
   <si>
     <t>MNLogit: 'Route outcomes after 3.08 years', table 0</t>
   </si>
@@ -49,7 +49,7 @@
     <t>rt_outcome</t>
   </si>
   <si>
-    <t>2026-06-14 15:09</t>
+    <t>2026-06-19 14:29</t>
   </si>
   <si>
     <t>2679</t>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>has_longer_term_rt</t>
+  </si>
+  <si>
+    <t>2026-06-19 14:30</t>
   </si>
   <si>
     <t>3032</t>
@@ -4683,7 +4686,7 @@
         <v>18</v>
       </c>
       <c r="E201" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="202" spans="1:6">
@@ -4694,13 +4697,13 @@
         <v>3</v>
       </c>
       <c r="C202" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="D202" t="s">
         <v>19</v>
       </c>
       <c r="E202" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="203" spans="1:6">
@@ -4711,13 +4714,13 @@
         <v>4</v>
       </c>
       <c r="C203" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D203" t="s">
         <v>20</v>
       </c>
       <c r="E203" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="204" spans="1:6">
@@ -4734,7 +4737,7 @@
         <v>21</v>
       </c>
       <c r="E204" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="205" spans="1:6">
@@ -4745,13 +4748,13 @@
         <v>6</v>
       </c>
       <c r="C205" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D205" t="s">
         <v>22</v>
       </c>
       <c r="E205" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="206" spans="1:6">
@@ -4768,7 +4771,7 @@
         <v>23</v>
       </c>
       <c r="E206" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="207" spans="1:6">
@@ -4779,7 +4782,7 @@
         <v>8</v>
       </c>
       <c r="C207" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D207" t="s">
         <v>24</v>
@@ -4790,7 +4793,7 @@
     </row>
     <row r="209" spans="1:7">
       <c r="A209" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="210" spans="1:7">
@@ -4861,7 +4864,7 @@
     </row>
     <row r="213" spans="1:7">
       <c r="A213" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B213">
         <v>-1.1</v>
@@ -4976,7 +4979,7 @@
     </row>
     <row r="219" spans="1:7">
       <c r="A219" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="220" spans="1:7">
@@ -5058,7 +5061,7 @@
     </row>
     <row r="224" spans="1:7">
       <c r="A224" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B224">
         <v>0.3</v>
@@ -5135,7 +5138,7 @@
     </row>
     <row r="229" spans="1:6">
       <c r="A229" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="230" spans="1:6">
@@ -5177,13 +5180,13 @@
         <v>2</v>
       </c>
       <c r="C232" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D232" t="s">
         <v>18</v>
       </c>
       <c r="E232" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="233" spans="1:6">
@@ -5194,13 +5197,13 @@
         <v>3</v>
       </c>
       <c r="C233" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="D233" t="s">
         <v>19</v>
       </c>
       <c r="E233" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="234" spans="1:6">
@@ -5211,13 +5214,13 @@
         <v>4</v>
       </c>
       <c r="C234" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D234" t="s">
         <v>20</v>
       </c>
       <c r="E234" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="235" spans="1:6">
@@ -5228,13 +5231,13 @@
         <v>5</v>
       </c>
       <c r="C235" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D235" t="s">
         <v>21</v>
       </c>
       <c r="E235" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="236" spans="1:6">
@@ -5245,13 +5248,13 @@
         <v>6</v>
       </c>
       <c r="C236" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D236" t="s">
         <v>22</v>
       </c>
       <c r="E236" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="237" spans="1:6">
@@ -5268,7 +5271,7 @@
         <v>23</v>
       </c>
       <c r="E237" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="238" spans="1:6">
@@ -5290,7 +5293,7 @@
     </row>
     <row r="240" spans="1:6">
       <c r="A240" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="241" spans="1:7">
@@ -5338,7 +5341,7 @@
     </row>
     <row r="243" spans="1:7">
       <c r="A243" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B243">
         <v>2.5</v>
@@ -5384,7 +5387,7 @@
     </row>
     <row r="245" spans="1:7">
       <c r="A245" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B245">
         <v>1.2</v>
@@ -5407,7 +5410,7 @@
     </row>
     <row r="247" spans="1:7">
       <c r="A247" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="248" spans="1:7">
@@ -5449,7 +5452,7 @@
     </row>
     <row r="250" spans="1:7">
       <c r="A250" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B250">
         <v>0</v>
@@ -5469,7 +5472,7 @@
     </row>
     <row r="251" spans="1:7">
       <c r="A251" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B251">
         <v>0</v>
@@ -5509,7 +5512,7 @@
     </row>
     <row r="254" spans="1:7">
       <c r="A254" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="255" spans="1:7">
@@ -5551,13 +5554,13 @@
         <v>2</v>
       </c>
       <c r="C257" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D257" t="s">
         <v>18</v>
       </c>
       <c r="E257" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="258" spans="1:8">
@@ -5568,13 +5571,13 @@
         <v>3</v>
       </c>
       <c r="C258" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="D258" t="s">
         <v>19</v>
       </c>
       <c r="E258" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="259" spans="1:8">
@@ -5585,13 +5588,13 @@
         <v>4</v>
       </c>
       <c r="C259" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D259" t="s">
         <v>20</v>
       </c>
       <c r="E259" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="260" spans="1:8">
@@ -5602,13 +5605,13 @@
         <v>5</v>
       </c>
       <c r="C260" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D260" t="s">
         <v>21</v>
       </c>
       <c r="E260" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="261" spans="1:8">
@@ -5619,13 +5622,13 @@
         <v>6</v>
       </c>
       <c r="C261" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D261" t="s">
         <v>22</v>
       </c>
       <c r="E261" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="262" spans="1:8">
@@ -5642,7 +5645,7 @@
         <v>23</v>
       </c>
       <c r="E262" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="263" spans="1:8">
@@ -5664,12 +5667,12 @@
     </row>
     <row r="265" spans="1:8">
       <c r="A265" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="266" spans="1:8">
       <c r="B266" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C266" s="1" t="s">
         <v>34</v>
@@ -5874,10 +5877,10 @@
     </row>
     <row r="274" spans="1:8">
       <c r="A274" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B274" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C274">
         <v>-0.2</v>
@@ -5978,10 +5981,10 @@
     </row>
     <row r="278" spans="1:8">
       <c r="A278" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B278" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C278">
         <v>-0.1</v>
@@ -6030,12 +6033,12 @@
     </row>
     <row r="281" spans="1:8">
       <c r="A281" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="282" spans="1:8">
       <c r="B282" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C282" s="1" t="s">
         <v>34</v>
@@ -6240,10 +6243,10 @@
     </row>
     <row r="290" spans="1:8">
       <c r="A290" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B290" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C290">
         <v>0.1</v>
@@ -6344,10 +6347,10 @@
     </row>
     <row r="294" spans="1:8">
       <c r="A294" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B294" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C294">
         <v>-0</v>
@@ -6396,12 +6399,12 @@
     </row>
     <row r="297" spans="1:8">
       <c r="A297" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="298" spans="1:8">
       <c r="B298" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C298" s="1" t="s">
         <v>34</v>
@@ -6606,10 +6609,10 @@
     </row>
     <row r="306" spans="1:8">
       <c r="A306" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B306" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C306">
         <v>-0.1</v>
@@ -6710,10 +6713,10 @@
     </row>
     <row r="310" spans="1:8">
       <c r="A310" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B310" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C310">
         <v>0.3</v>
@@ -6762,12 +6765,12 @@
     </row>
     <row r="313" spans="1:8">
       <c r="A313" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="314" spans="1:8">
       <c r="B314" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C314" s="1" t="s">
         <v>34</v>
@@ -6972,10 +6975,10 @@
     </row>
     <row r="322" spans="1:8">
       <c r="A322" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B322" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C322">
         <v>0.1</v>
@@ -7076,10 +7079,10 @@
     </row>
     <row r="326" spans="1:8">
       <c r="A326" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B326" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C326">
         <v>0.1</v>
@@ -7128,12 +7131,12 @@
     </row>
     <row r="329" spans="1:8">
       <c r="A329" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="330" spans="1:8">
       <c r="B330" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C330" s="1" t="s">
         <v>34</v>
@@ -7338,10 +7341,10 @@
     </row>
     <row r="338" spans="1:8">
       <c r="A338" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B338" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C338">
         <v>-0</v>
@@ -7442,10 +7445,10 @@
     </row>
     <row r="342" spans="1:8">
       <c r="A342" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B342" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C342">
         <v>0.1</v>
@@ -7494,12 +7497,12 @@
     </row>
     <row r="345" spans="1:8">
       <c r="A345" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="346" spans="1:8">
       <c r="B346" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C346" s="1" t="s">
         <v>34</v>
@@ -7704,10 +7707,10 @@
     </row>
     <row r="354" spans="1:8">
       <c r="A354" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B354" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C354">
         <v>-0.4</v>
@@ -7808,10 +7811,10 @@
     </row>
     <row r="358" spans="1:8">
       <c r="A358" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B358" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C358">
         <v>-0.5</v>
@@ -7860,7 +7863,7 @@
     </row>
     <row r="361" spans="1:8">
       <c r="A361" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="362" spans="1:8">
@@ -7945,7 +7948,7 @@
     <row r="366" spans="1:8">
       <c r="A366" s="1"/>
       <c r="B366" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C366">
         <v>0.1</v>
@@ -8020,7 +8023,7 @@
     <row r="370" spans="1:7">
       <c r="A370" s="1"/>
       <c r="B370" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C370">
         <v>0.2</v>
@@ -8130,7 +8133,7 @@
     </row>
     <row r="376" spans="1:7">
       <c r="A376" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B376" s="1" t="s">
         <v>40</v>
@@ -8190,7 +8193,7 @@
     <row r="379" spans="1:7">
       <c r="A379" s="1"/>
       <c r="B379" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C379">
         <v>0</v>
@@ -8271,7 +8274,7 @@
     <row r="383" spans="1:7">
       <c r="A383" s="1"/>
       <c r="B383" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C383">
         <v>0.4</v>
@@ -8384,7 +8387,7 @@
     </row>
     <row r="389" spans="1:7">
       <c r="A389" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B389" s="1" t="s">
         <v>40</v>
@@ -8447,7 +8450,7 @@
     <row r="392" spans="1:7">
       <c r="A392" s="1"/>
       <c r="B392" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C392">
         <v>0.7</v>
@@ -8522,7 +8525,7 @@
     <row r="396" spans="1:7">
       <c r="A396" s="1"/>
       <c r="B396" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C396">
         <v>0.7</v>
@@ -8635,7 +8638,7 @@
     </row>
     <row r="402" spans="1:7">
       <c r="A402" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B402" s="1" t="s">
         <v>40</v>
@@ -8695,7 +8698,7 @@
     <row r="405" spans="1:7">
       <c r="A405" s="1"/>
       <c r="B405" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C405">
         <v>0.5</v>
@@ -8767,7 +8770,7 @@
     <row r="409" spans="1:7">
       <c r="A409" s="1"/>
       <c r="B409" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C409">
         <v>0.3</v>
@@ -8877,7 +8880,7 @@
     </row>
     <row r="415" spans="1:7">
       <c r="A415" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B415" s="1" t="s">
         <v>40</v>
@@ -8943,7 +8946,7 @@
     <row r="418" spans="1:7">
       <c r="A418" s="1"/>
       <c r="B418" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C418">
         <v>0.5</v>
@@ -9021,7 +9024,7 @@
     <row r="422" spans="1:7">
       <c r="A422" s="1"/>
       <c r="B422" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C422">
         <v>0.9</v>
@@ -9197,7 +9200,7 @@
     <row r="431" spans="1:7">
       <c r="A431" s="1"/>
       <c r="B431" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C431">
         <v>0.2</v>
@@ -9275,7 +9278,7 @@
     <row r="435" spans="1:7">
       <c r="A435" s="1"/>
       <c r="B435" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C435">
         <v>0</v>

</xml_diff>

<commit_message>
Style improvements to visualisation footer text.
</commit_message>
<xml_diff>
--- a/assets_output/09_logistic_regression_blocks.xlsx
+++ b/assets_output/09_logistic_regression_blocks.xlsx
@@ -49,7 +49,7 @@
     <t>rt_outcome</t>
   </si>
   <si>
-    <t>2026-06-19 14:50</t>
+    <t>2026-06-19 14:59</t>
   </si>
   <si>
     <t>2679</t>
@@ -313,7 +313,7 @@
     <t>has_longer_term_rt</t>
   </si>
   <si>
-    <t>2026-06-19 14:51</t>
+    <t>2026-06-19 15:00</t>
   </si>
   <si>
     <t>3032</t>

</xml_diff>

<commit_message>
Fixed excel output (number format) .. now including column G!
</commit_message>
<xml_diff>
--- a/assets_output/09_logistic_regression_blocks.xlsx
+++ b/assets_output/09_logistic_regression_blocks.xlsx
@@ -49,7 +49,7 @@
     <t>rt_outcome</t>
   </si>
   <si>
-    <t>2026-06-20 11:53</t>
+    <t>2026-06-20 12:03</t>
   </si>
   <si>
     <t>2679</t>
@@ -208,9 +208,6 @@
     <t>cli_outcome</t>
   </si>
   <si>
-    <t>2026-06-20 11:54</t>
-  </si>
-  <si>
     <t>2014</t>
   </si>
   <si>
@@ -269,6 +266,9 @@
   </si>
   <si>
     <t>multiple_returns</t>
+  </si>
+  <si>
+    <t>2026-06-20 12:04</t>
   </si>
   <si>
     <t>3015</t>
@@ -855,7 +855,7 @@
   <dimension ref="A1:H476"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="7" width="9.140625" style="1"/>
+    <col min="3" max="8" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1063,7 +1063,7 @@
       <c r="G14" s="1">
         <v>-1.11392903337809</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="1">
         <v>-0.6771811836907633</v>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       <c r="G15" s="1">
         <v>-0.4664249767471592</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="1">
         <v>0.01388151312686606</v>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
       <c r="G16" s="1">
         <v>0.08279480070465725</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="1">
         <v>0.5198881519044269</v>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       <c r="G17" s="1">
         <v>-0.9239845564630997</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="1">
         <v>-0.1923814052085897</v>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       <c r="G18" s="1">
         <v>-0.7284895018228333</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="1">
         <v>0.4767695563220496</v>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
       <c r="G19" s="1">
         <v>0.7365420173661663</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="1">
         <v>1.34989440607928</v>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       <c r="G20" s="1">
         <v>0.04728124236257084</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="1">
         <v>0.4849791568365172</v>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       <c r="G21" s="1">
         <v>1.050661769717664</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="1">
         <v>1.483762529884471</v>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       <c r="G22" s="1">
         <v>0.201091380258715</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="1">
         <v>0.7789886830308901</v>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       <c r="G23" s="1">
         <v>0.5236482076952025</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="1">
         <v>3.495677134365566</v>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
       <c r="G24" s="1">
         <v>0.02136272894230934</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="1">
         <v>0.8032696084855746</v>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       <c r="G28" s="1">
         <v>-1.598398172647587</v>
       </c>
-      <c r="H28">
+      <c r="H28" s="1">
         <v>-1.115806990223457</v>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       <c r="G29" s="1">
         <v>-0.6076771548383374</v>
       </c>
-      <c r="H29">
+      <c r="H29" s="1">
         <v>-0.0846235192558179</v>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       <c r="G30" s="1">
         <v>-0.009359675379155691</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="1">
         <v>0.4525063299653923</v>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       <c r="G31" s="1">
         <v>-1.311202228878892</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="1">
         <v>-0.4091390632618893</v>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       <c r="G32" s="1">
         <v>-0.3906379681625919</v>
       </c>
-      <c r="H32">
+      <c r="H32" s="1">
         <v>0.8205279544400883</v>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       <c r="G33" s="1">
         <v>0.9834857793138327</v>
       </c>
-      <c r="H33">
+      <c r="H33" s="1">
         <v>1.601909089934065</v>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       <c r="G34" s="1">
         <v>-0.1081427162185326</v>
       </c>
-      <c r="H34">
+      <c r="H34" s="1">
         <v>0.3533904765169871</v>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       <c r="G35" s="1">
         <v>1.483541591110296</v>
       </c>
-      <c r="H35">
+      <c r="H35" s="1">
         <v>1.952539403950829</v>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       <c r="G36" s="1">
         <v>0.8201709235385017</v>
       </c>
-      <c r="H36">
+      <c r="H36" s="1">
         <v>1.387319471441722</v>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       <c r="G37" s="1">
         <v>0.7101315293755073</v>
       </c>
-      <c r="H37">
+      <c r="H37" s="1">
         <v>3.701468415464758</v>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       <c r="G38" s="1">
         <v>-0.1622614325075197</v>
       </c>
-      <c r="H38">
+      <c r="H38" s="1">
         <v>0.6640108904397559</v>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       <c r="G42" s="1">
         <v>-4.590412142661291</v>
       </c>
-      <c r="H42">
+      <c r="H42" s="1">
         <v>-3.083112121701626</v>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       <c r="G43" s="1">
         <v>-1.27002330243478</v>
       </c>
-      <c r="H43">
+      <c r="H43" s="1">
         <v>0.3175047081542241</v>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       <c r="G44" s="1">
         <v>-1.742754103359455</v>
       </c>
-      <c r="H44">
+      <c r="H44" s="1">
         <v>-0.07616710704500573</v>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
       <c r="G45" s="1">
         <v>-1.57490143462012</v>
       </c>
-      <c r="H45">
+      <c r="H45" s="1">
         <v>0.8730840651048752</v>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
       <c r="G46" s="1">
         <v>-0.2391325064177163</v>
       </c>
-      <c r="H46">
+      <c r="H46" s="1">
         <v>2.311771029488853</v>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       <c r="G47" s="1">
         <v>-0.8400555367908615</v>
       </c>
-      <c r="H47">
+      <c r="H47" s="1">
         <v>0.9939348365493195</v>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="G48" s="1">
         <v>0.1439029390041684</v>
       </c>
-      <c r="H48">
+      <c r="H48" s="1">
         <v>1.351763038172491</v>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       <c r="G49" s="1">
         <v>1.164531804614537</v>
       </c>
-      <c r="H49">
+      <c r="H49" s="1">
         <v>2.587692101413705</v>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       <c r="G50" s="1">
         <v>-1.019312160346784</v>
       </c>
-      <c r="H50">
+      <c r="H50" s="1">
         <v>0.6804843090684729</v>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       <c r="G51" s="1">
         <v>0.6708046202848363</v>
       </c>
-      <c r="H51">
+      <c r="H51" s="1">
         <v>4.960468528318827</v>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       <c r="G52" s="1">
         <v>-2.379952731895911</v>
       </c>
-      <c r="H52">
+      <c r="H52" s="1">
         <v>0.5639181848985116</v>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
         <v>18</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -2701,13 +2701,13 @@
         <v>3</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -2718,13 +2718,13 @@
         <v>4</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -2735,13 +2735,13 @@
         <v>5</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -2752,13 +2752,13 @@
         <v>6</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -2775,7 +2775,7 @@
         <v>23</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -2786,7 +2786,7 @@
         <v>8</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D99" s="1" t="s">
         <v>24</v>
@@ -2797,12 +2797,12 @@
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="102" spans="1:8">
       <c r="B102" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C102" s="2" t="s">
         <v>34</v>
@@ -2845,7 +2845,7 @@
       <c r="G103" s="1">
         <v>-1.581671125626535</v>
       </c>
-      <c r="H103">
+      <c r="H103" s="1">
         <v>-1.121933421239041</v>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       <c r="G104" s="1">
         <v>0.09821225139456244</v>
       </c>
-      <c r="H104">
+      <c r="H104" s="1">
         <v>0.5630220212008613</v>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       <c r="G105" s="1">
         <v>-1.105158534854958</v>
       </c>
-      <c r="H105">
+      <c r="H105" s="1">
         <v>-0.2719567335956136</v>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
       <c r="G106" s="1">
         <v>-0.7431440666727596</v>
       </c>
-      <c r="H106">
+      <c r="H106" s="1">
         <v>0.4894810949225405</v>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
       <c r="G107" s="1">
         <v>0.7804091716324164</v>
       </c>
-      <c r="H107">
+      <c r="H107" s="1">
         <v>1.421845837535434</v>
       </c>
     </row>
@@ -2975,7 +2975,7 @@
       <c r="G108" s="1">
         <v>0.06152846867379258</v>
       </c>
-      <c r="H108">
+      <c r="H108" s="1">
         <v>0.5254846845735226</v>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       <c r="G109" s="1">
         <v>1.09511987964771</v>
       </c>
-      <c r="H109">
+      <c r="H109" s="1">
         <v>1.553474525821898</v>
       </c>
     </row>
@@ -3027,7 +3027,7 @@
       <c r="G110" s="1">
         <v>0.2572075455024447</v>
       </c>
-      <c r="H110">
+      <c r="H110" s="1">
         <v>0.8689035141718615</v>
       </c>
     </row>
@@ -3053,18 +3053,18 @@
       <c r="G111" s="1">
         <v>0.5514154012494417</v>
       </c>
-      <c r="H111">
+      <c r="H111" s="1">
         <v>3.577640313321367</v>
       </c>
     </row>
     <row r="113" spans="1:8">
       <c r="A113" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="114" spans="1:8">
       <c r="B114" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C114" s="2" t="s">
         <v>34</v>
@@ -3107,7 +3107,7 @@
       <c r="G115" s="1">
         <v>-2.26094286510595</v>
       </c>
-      <c r="H115">
+      <c r="H115" s="1">
         <v>-1.703790596333637</v>
       </c>
     </row>
@@ -3133,7 +3133,7 @@
       <c r="G116" s="1">
         <v>0.09977619639470781</v>
       </c>
-      <c r="H116">
+      <c r="H116" s="1">
         <v>0.6340541049345748</v>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       <c r="G117" s="1">
         <v>-1.445298367343927</v>
       </c>
-      <c r="H117">
+      <c r="H117" s="1">
         <v>-0.320375812927729</v>
       </c>
     </row>
@@ -3185,7 +3185,7 @@
       <c r="G118" s="1">
         <v>-0.5552189959505973</v>
       </c>
-      <c r="H118">
+      <c r="H118" s="1">
         <v>0.7971064393036733</v>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       <c r="G119" s="1">
         <v>1.057537946935777</v>
       </c>
-      <c r="H119">
+      <c r="H119" s="1">
         <v>1.742491397233148</v>
       </c>
     </row>
@@ -3237,7 +3237,7 @@
       <c r="G120" s="1">
         <v>-0.4405542135482299</v>
       </c>
-      <c r="H120">
+      <c r="H120" s="1">
         <v>0.113856668556694</v>
       </c>
     </row>
@@ -3263,7 +3263,7 @@
       <c r="G121" s="1">
         <v>1.161560996922351</v>
       </c>
-      <c r="H121">
+      <c r="H121" s="1">
         <v>1.709458263052691</v>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
       <c r="G122" s="1">
         <v>0.9176530279087538</v>
       </c>
-      <c r="H122">
+      <c r="H122" s="1">
         <v>1.552383594767749</v>
       </c>
     </row>
@@ -3315,18 +3315,18 @@
       <c r="G123" s="1">
         <v>0.4147109040290966</v>
       </c>
-      <c r="H123">
+      <c r="H123" s="1">
         <v>3.56721682068298</v>
       </c>
     </row>
     <row r="125" spans="1:8">
       <c r="A125" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="126" spans="1:8">
       <c r="B126" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C126" s="2" t="s">
         <v>34</v>
@@ -3369,7 +3369,7 @@
       <c r="G127" s="1">
         <v>-4.651449608929791</v>
       </c>
-      <c r="H127">
+      <c r="H127" s="1">
         <v>-3.125417455077427</v>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       <c r="G128" s="1">
         <v>-2.010675540612974</v>
       </c>
-      <c r="H128">
+      <c r="H128" s="1">
         <v>-0.05662752269617033</v>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       <c r="G129" s="1">
         <v>-1.983359913220259</v>
       </c>
-      <c r="H129">
+      <c r="H129" s="1">
         <v>0.9658182630324635</v>
       </c>
     </row>
@@ -3447,7 +3447,7 @@
       <c r="G130" s="1">
         <v>-0.8141782442142619</v>
       </c>
-      <c r="H130">
+      <c r="H130" s="1">
         <v>2.188265962122714</v>
       </c>
     </row>
@@ -3473,7 +3473,7 @@
       <c r="G131" s="1">
         <v>-0.4763501192047371</v>
       </c>
-      <c r="H131">
+      <c r="H131" s="1">
         <v>1.506320001443703</v>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="G132" s="1">
         <v>-0.2109480295578882</v>
       </c>
-      <c r="H132">
+      <c r="H132" s="1">
         <v>1.182250792286782</v>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
       <c r="G133" s="1">
         <v>0.5626440109166015</v>
       </c>
-      <c r="H133">
+      <c r="H133" s="1">
         <v>2.06934081441574</v>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       <c r="G134" s="1">
         <v>-0.9479014751812982</v>
       </c>
-      <c r="H134">
+      <c r="H134" s="1">
         <v>1.035544504843304</v>
       </c>
     </row>
@@ -3577,13 +3577,13 @@
       <c r="G135" s="1">
         <v>-0.1724693582507544</v>
       </c>
-      <c r="H135">
+      <c r="H135" s="1">
         <v>4.777935751991526</v>
       </c>
     </row>
     <row r="137" spans="1:8">
       <c r="A137" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="138" spans="1:8">
@@ -4151,7 +4151,7 @@
     </row>
     <row r="167" spans="1:7">
       <c r="A167" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -4176,7 +4176,7 @@
         <v>1</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D169" s="1" t="s">
         <v>17</v>
@@ -4193,7 +4193,7 @@
         <v>2</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D170" s="1" t="s">
         <v>18</v>
@@ -4210,7 +4210,7 @@
         <v>3</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="D171" s="1" t="s">
         <v>19</v>
@@ -4295,7 +4295,7 @@
         <v>8</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D176" s="1" t="s">
         <v>24</v>
@@ -4679,7 +4679,7 @@
         <v>1</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D200" s="1" t="s">
         <v>17</v>
@@ -4713,7 +4713,7 @@
         <v>3</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="D202" s="1" t="s">
         <v>19</v>
@@ -5179,7 +5179,7 @@
         <v>1</v>
       </c>
       <c r="C231" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D231" s="1" t="s">
         <v>17</v>
@@ -5213,7 +5213,7 @@
         <v>3</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="D233" s="1" t="s">
         <v>19</v>
@@ -5587,7 +5587,7 @@
         <v>3</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="D258" s="1" t="s">
         <v>19</v>
@@ -5672,7 +5672,7 @@
         <v>8</v>
       </c>
       <c r="C263" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D263" s="1" t="s">
         <v>24</v>
@@ -5731,7 +5731,7 @@
       <c r="G267" s="1">
         <v>-0.3794521339112729</v>
       </c>
-      <c r="H267">
+      <c r="H267" s="1">
         <v>0.05596069615941091</v>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       <c r="G268" s="1">
         <v>-0.4156794261977594</v>
       </c>
-      <c r="H268">
+      <c r="H268" s="1">
         <v>0.008212463020749405</v>
       </c>
     </row>
@@ -5783,7 +5783,7 @@
       <c r="G269" s="1">
         <v>-0.09855550044876138</v>
       </c>
-      <c r="H269">
+      <c r="H269" s="1">
         <v>0.2852048773364834</v>
       </c>
     </row>
@@ -5809,7 +5809,7 @@
       <c r="G270" s="1">
         <v>-0.5206101709821805</v>
       </c>
-      <c r="H270">
+      <c r="H270" s="1">
         <v>0.04045529280377202</v>
       </c>
     </row>
@@ -5835,7 +5835,7 @@
       <c r="G271" s="1">
         <v>-0.5178652812497002</v>
       </c>
-      <c r="H271">
+      <c r="H271" s="1">
         <v>0.282641141164032</v>
       </c>
     </row>
@@ -5861,7 +5861,7 @@
       <c r="G272" s="1">
         <v>-0.592490250309573</v>
       </c>
-      <c r="H272">
+      <c r="H272" s="1">
         <v>0.2422490531489189</v>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
       <c r="G273" s="1">
         <v>-0.4076298473186334</v>
       </c>
-      <c r="H273">
+      <c r="H273" s="1">
         <v>0.258787783388101</v>
       </c>
     </row>
@@ -5913,7 +5913,7 @@
       <c r="G274" s="1">
         <v>-0.3628869222050291</v>
       </c>
-      <c r="H274">
+      <c r="H274" s="1">
         <v>0.5725779932168049</v>
       </c>
     </row>
@@ -5939,7 +5939,7 @@
       <c r="G275" s="1">
         <v>0.2569037196486199</v>
       </c>
-      <c r="H275">
+      <c r="H275" s="1">
         <v>0.8457558249120503</v>
       </c>
     </row>
@@ -5965,7 +5965,7 @@
       <c r="G276" s="1">
         <v>-0.08241003193804454</v>
       </c>
-      <c r="H276">
+      <c r="H276" s="1">
         <v>0.2994432408921167</v>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       <c r="G277" s="1">
         <v>0.02913405936958183</v>
       </c>
-      <c r="H277">
+      <c r="H277" s="1">
         <v>0.4164607320931782</v>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
       <c r="G278" s="1">
         <v>0.6636036815215647</v>
       </c>
-      <c r="H278">
+      <c r="H278" s="1">
         <v>1.053377552986486</v>
       </c>
     </row>
@@ -6043,7 +6043,7 @@
       <c r="G279" s="1">
         <v>-0.2264007150358374</v>
       </c>
-      <c r="H279">
+      <c r="H279" s="1">
         <v>0.3287318803315753</v>
       </c>
     </row>
@@ -6069,7 +6069,7 @@
       <c r="G280" s="1">
         <v>0.2509095883644255</v>
       </c>
-      <c r="H280">
+      <c r="H280" s="1">
         <v>2.365493653693948</v>
       </c>
     </row>
@@ -6095,7 +6095,7 @@
       <c r="G281" s="1">
         <v>-0.1313914841385387</v>
       </c>
-      <c r="H281">
+      <c r="H281" s="1">
         <v>0.3971902230541606</v>
       </c>
     </row>
@@ -6121,7 +6121,7 @@
       <c r="G282" s="1">
         <v>0.0928326932544668</v>
       </c>
-      <c r="H282">
+      <c r="H282" s="1">
         <v>0.8218305198931841</v>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       <c r="G286" s="1">
         <v>-2.029965583019055</v>
       </c>
-      <c r="H286">
+      <c r="H286" s="1">
         <v>-1.470084922694495</v>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       <c r="G287" s="1">
         <v>-0.7523918254036385</v>
       </c>
-      <c r="H287">
+      <c r="H287" s="1">
         <v>-0.2543621368008436</v>
       </c>
     </row>
@@ -6227,7 +6227,7 @@
       <c r="G288" s="1">
         <v>0.2305917466235909</v>
       </c>
-      <c r="H288">
+      <c r="H288" s="1">
         <v>0.6562999672258583</v>
       </c>
     </row>
@@ -6253,7 +6253,7 @@
       <c r="G289" s="1">
         <v>-0.5730547224899674</v>
       </c>
-      <c r="H289">
+      <c r="H289" s="1">
         <v>0.1239337246814425</v>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       <c r="G290" s="1">
         <v>-0.3647661217938782</v>
       </c>
-      <c r="H290">
+      <c r="H290" s="1">
         <v>0.5161779499616461</v>
       </c>
     </row>
@@ -6305,7 +6305,7 @@
       <c r="G291" s="1">
         <v>-0.6101141260653213</v>
       </c>
-      <c r="H291">
+      <c r="H291" s="1">
         <v>0.4599743893740868</v>
       </c>
     </row>
@@ -6331,7 +6331,7 @@
       <c r="G292" s="1">
         <v>-1.173265044696065</v>
       </c>
-      <c r="H292">
+      <c r="H292" s="1">
         <v>-0.2352943097830613</v>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       <c r="G293" s="1">
         <v>-0.9061301887400135</v>
       </c>
-      <c r="H293">
+      <c r="H293" s="1">
         <v>0.2917793033203441</v>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       <c r="G294" s="1">
         <v>0.8482745320418015</v>
       </c>
-      <c r="H294">
+      <c r="H294" s="1">
         <v>1.442096917649641</v>
       </c>
     </row>
@@ -6409,7 +6409,7 @@
       <c r="G295" s="1">
         <v>0.09510166709235848</v>
       </c>
-      <c r="H295">
+      <c r="H295" s="1">
         <v>0.5157075113464218</v>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       <c r="G296" s="1">
         <v>0.06667682371058628</v>
       </c>
-      <c r="H296">
+      <c r="H296" s="1">
         <v>0.5225732684393821</v>
       </c>
     </row>
@@ -6461,7 +6461,7 @@
       <c r="G297" s="1">
         <v>1.895775871206949</v>
       </c>
-      <c r="H297">
+      <c r="H297" s="1">
         <v>2.369129669327319</v>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       <c r="G298" s="1">
         <v>0.5344773274419343</v>
       </c>
-      <c r="H298">
+      <c r="H298" s="1">
         <v>1.082229491680292</v>
       </c>
     </row>
@@ -6513,7 +6513,7 @@
       <c r="G299" s="1">
         <v>0.6153211839312183</v>
       </c>
-      <c r="H299">
+      <c r="H299" s="1">
         <v>2.736269407437578</v>
       </c>
     </row>
@@ -6539,7 +6539,7 @@
       <c r="G300" s="1">
         <v>-0.1736908324032717</v>
       </c>
-      <c r="H300">
+      <c r="H300" s="1">
         <v>0.4179751144470288</v>
       </c>
     </row>
@@ -6565,7 +6565,7 @@
       <c r="G301" s="1">
         <v>0.06460931570213491</v>
       </c>
-      <c r="H301">
+      <c r="H301" s="1">
         <v>0.8304754246572181</v>
       </c>
     </row>
@@ -6619,7 +6619,7 @@
       <c r="G305" s="1">
         <v>-2.072725186876687</v>
       </c>
-      <c r="H305">
+      <c r="H305" s="1">
         <v>-1.460896647553666</v>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       <c r="G306" s="1">
         <v>-0.3405916219352946</v>
       </c>
-      <c r="H306">
+      <c r="H306" s="1">
         <v>0.1897202485915027</v>
       </c>
     </row>
@@ -6671,7 +6671,7 @@
       <c r="G307" s="1">
         <v>-0.04716994659839932</v>
       </c>
-      <c r="H307">
+      <c r="H307" s="1">
         <v>0.4316558923622377</v>
       </c>
     </row>
@@ -6697,7 +6697,7 @@
       <c r="G308" s="1">
         <v>-0.5414807457307159</v>
       </c>
-      <c r="H308">
+      <c r="H308" s="1">
         <v>0.2181943098687102</v>
       </c>
     </row>
@@ -6723,7 +6723,7 @@
       <c r="G309" s="1">
         <v>-0.3346749806920611</v>
       </c>
-      <c r="H309">
+      <c r="H309" s="1">
         <v>0.6225128769362706</v>
       </c>
     </row>
@@ -6749,7 +6749,7 @@
       <c r="G310" s="1">
         <v>-1.070329688994984</v>
       </c>
-      <c r="H310">
+      <c r="H310" s="1">
         <v>0.1611247705406285</v>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       <c r="G311" s="1">
         <v>-0.382400541654449</v>
       </c>
-      <c r="H311">
+      <c r="H311" s="1">
         <v>0.5109474205583086</v>
       </c>
     </row>
@@ -6801,7 +6801,7 @@
       <c r="G312" s="1">
         <v>-0.2232518259586685</v>
       </c>
-      <c r="H312">
+      <c r="H312" s="1">
         <v>0.9327930429342112</v>
       </c>
     </row>
@@ -6827,7 +6827,7 @@
       <c r="G313" s="1">
         <v>0.3796587802912924</v>
       </c>
-      <c r="H313">
+      <c r="H313" s="1">
         <v>1.055820429376243</v>
       </c>
     </row>
@@ -6853,7 +6853,7 @@
       <c r="G314" s="1">
         <v>-0.1095286321140161</v>
       </c>
-      <c r="H314">
+      <c r="H314" s="1">
         <v>0.3627804638057345</v>
       </c>
     </row>
@@ -6879,7 +6879,7 @@
       <c r="G315" s="1">
         <v>0.01714843807045363</v>
       </c>
-      <c r="H315">
+      <c r="H315" s="1">
         <v>0.5286652165240471</v>
       </c>
     </row>
@@ -6905,7 +6905,7 @@
       <c r="G316" s="1">
         <v>1.390289901573426</v>
       </c>
-      <c r="H316">
+      <c r="H316" s="1">
         <v>1.897608378770266</v>
       </c>
     </row>
@@ -6931,7 +6931,7 @@
       <c r="G317" s="1">
         <v>-0.1287881369037527</v>
       </c>
-      <c r="H317">
+      <c r="H317" s="1">
         <v>0.5104473116702856</v>
       </c>
     </row>
@@ -6957,7 +6957,7 @@
       <c r="G318" s="1">
         <v>0.3917152749969173</v>
       </c>
-      <c r="H318">
+      <c r="H318" s="1">
         <v>2.560632861239616</v>
       </c>
     </row>
@@ -6983,7 +6983,7 @@
       <c r="G319" s="1">
         <v>-0.06196136672496927</v>
       </c>
-      <c r="H319">
+      <c r="H319" s="1">
         <v>0.5723969009635295</v>
       </c>
     </row>
@@ -7009,7 +7009,7 @@
       <c r="G320" s="1">
         <v>0.2460957029449067</v>
       </c>
-      <c r="H320">
+      <c r="H320" s="1">
         <v>1.051289388167086</v>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       <c r="G324" s="1">
         <v>-1.779681354985243</v>
       </c>
-      <c r="H324">
+      <c r="H324" s="1">
         <v>-1.203673209740966</v>
       </c>
     </row>
@@ -7089,7 +7089,7 @@
       <c r="G325" s="1">
         <v>-0.7127365325249728</v>
       </c>
-      <c r="H325">
+      <c r="H325" s="1">
         <v>-0.1554162212376664</v>
       </c>
     </row>
@@ -7115,7 +7115,7 @@
       <c r="G326" s="1">
         <v>0.02492089707416853</v>
       </c>
-      <c r="H326">
+      <c r="H326" s="1">
         <v>0.4969478061980688</v>
       </c>
     </row>
@@ -7141,7 +7141,7 @@
       <c r="G327" s="1">
         <v>-0.5137537833940388</v>
       </c>
-      <c r="H327">
+      <c r="H327" s="1">
         <v>0.2349713644088363</v>
       </c>
     </row>
@@ -7167,7 +7167,7 @@
       <c r="G328" s="1">
         <v>-0.2593570436178049</v>
       </c>
-      <c r="H328">
+      <c r="H328" s="1">
         <v>0.6827400439911467</v>
       </c>
     </row>
@@ -7193,7 +7193,7 @@
       <c r="G329" s="1">
         <v>-0.771983646886419</v>
       </c>
-      <c r="H329">
+      <c r="H329" s="1">
         <v>0.4394190304625612</v>
       </c>
     </row>
@@ -7219,7 +7219,7 @@
       <c r="G330" s="1">
         <v>-1.381128981040567</v>
       </c>
-      <c r="H330">
+      <c r="H330" s="1">
         <v>-0.3017835157078526</v>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
       <c r="G331" s="1">
         <v>-0.3377962619885364</v>
       </c>
-      <c r="H331">
+      <c r="H331" s="1">
         <v>0.8166958990011259</v>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       <c r="G332" s="1">
         <v>0.8143774989642329</v>
       </c>
-      <c r="H332">
+      <c r="H332" s="1">
         <v>1.447641279784983</v>
       </c>
     </row>
@@ -7297,7 +7297,7 @@
       <c r="G333" s="1">
         <v>-0.260938305050137</v>
       </c>
-      <c r="H333">
+      <c r="H333" s="1">
         <v>0.2120565023667073</v>
       </c>
     </row>
@@ -7323,7 +7323,7 @@
       <c r="G334" s="1">
         <v>-0.1999110807604748</v>
       </c>
-      <c r="H334">
+      <c r="H334" s="1">
         <v>0.2907875932124501</v>
       </c>
     </row>
@@ -7349,7 +7349,7 @@
       <c r="G335" s="1">
         <v>1.16081756745314</v>
       </c>
-      <c r="H335">
+      <c r="H335" s="1">
         <v>1.65861368521251</v>
       </c>
     </row>
@@ -7375,7 +7375,7 @@
       <c r="G336" s="1">
         <v>0.8361674612182191</v>
       </c>
-      <c r="H336">
+      <c r="H336" s="1">
         <v>1.415019414558038</v>
       </c>
     </row>
@@ -7401,7 +7401,7 @@
       <c r="G337" s="1">
         <v>0.07503980290788737</v>
       </c>
-      <c r="H337">
+      <c r="H337" s="1">
         <v>2.326292122397795</v>
       </c>
     </row>
@@ -7427,7 +7427,7 @@
       <c r="G338" s="1">
         <v>0.1016957884901405</v>
       </c>
-      <c r="H338">
+      <c r="H338" s="1">
         <v>0.7424539501964886</v>
       </c>
     </row>
@@ -7453,7 +7453,7 @@
       <c r="G339" s="1">
         <v>-0.236752523531176</v>
       </c>
-      <c r="H339">
+      <c r="H339" s="1">
         <v>0.6337690560963747</v>
       </c>
     </row>
@@ -7507,7 +7507,7 @@
       <c r="G343" s="1">
         <v>-1.7832611939023</v>
       </c>
-      <c r="H343">
+      <c r="H343" s="1">
         <v>-1.186612231126567</v>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
       <c r="G344" s="1">
         <v>-0.5406015896630854</v>
       </c>
-      <c r="H344">
+      <c r="H344" s="1">
         <v>0.03097531535405146</v>
       </c>
     </row>
@@ -7559,7 +7559,7 @@
       <c r="G345" s="1">
         <v>0.1270387599356181</v>
       </c>
-      <c r="H345">
+      <c r="H345" s="1">
         <v>0.6212667389029632</v>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       <c r="G346" s="1">
         <v>-0.8381303894055891</v>
       </c>
-      <c r="H346">
+      <c r="H346" s="1">
         <v>-0.01840949957910193</v>
       </c>
     </row>
@@ -7611,7 +7611,7 @@
       <c r="G347" s="1">
         <v>-0.4237964386129014</v>
       </c>
-      <c r="H347">
+      <c r="H347" s="1">
         <v>0.5767915293081115</v>
       </c>
     </row>
@@ -7637,7 +7637,7 @@
       <c r="G348" s="1">
         <v>-0.4531655650997795</v>
       </c>
-      <c r="H348">
+      <c r="H348" s="1">
         <v>0.6760699267891392</v>
       </c>
     </row>
@@ -7663,7 +7663,7 @@
       <c r="G349" s="1">
         <v>-1.032061481682584</v>
       </c>
-      <c r="H349">
+      <c r="H349" s="1">
         <v>0.002354701984092156</v>
       </c>
     </row>
@@ -7689,7 +7689,7 @@
       <c r="G350" s="1">
         <v>-0.7211615688475324</v>
       </c>
-      <c r="H350">
+      <c r="H350" s="1">
         <v>0.5910706460996578</v>
       </c>
     </row>
@@ -7715,7 +7715,7 @@
       <c r="G351" s="1">
         <v>0.9001411363603826</v>
       </c>
-      <c r="H351">
+      <c r="H351" s="1">
         <v>1.555911414664031</v>
       </c>
     </row>
@@ -7741,7 +7741,7 @@
       <c r="G352" s="1">
         <v>-0.09535135922127466</v>
       </c>
-      <c r="H352">
+      <c r="H352" s="1">
         <v>0.4010403355315284</v>
       </c>
     </row>
@@ -7767,7 +7767,7 @@
       <c r="G353" s="1">
         <v>-0.1138148149619644</v>
       </c>
-      <c r="H353">
+      <c r="H353" s="1">
         <v>0.4057781958152997</v>
       </c>
     </row>
@@ -7793,7 +7793,7 @@
       <c r="G354" s="1">
         <v>0.7179174510773059</v>
       </c>
-      <c r="H354">
+      <c r="H354" s="1">
         <v>1.22715333600319</v>
       </c>
     </row>
@@ -7819,7 +7819,7 @@
       <c r="G355" s="1">
         <v>0.1780476598988924</v>
       </c>
-      <c r="H355">
+      <c r="H355" s="1">
         <v>0.8241542965455424</v>
       </c>
     </row>
@@ -7845,7 +7845,7 @@
       <c r="G356" s="1">
         <v>-0.4319139815820435</v>
       </c>
-      <c r="H356">
+      <c r="H356" s="1">
         <v>1.983054500026549</v>
       </c>
     </row>
@@ -7871,7 +7871,7 @@
       <c r="G357" s="1">
         <v>-0.1643150917220104</v>
       </c>
-      <c r="H357">
+      <c r="H357" s="1">
         <v>0.5189407390004216</v>
       </c>
     </row>
@@ -7897,7 +7897,7 @@
       <c r="G358" s="1">
         <v>-0.003782097928405614</v>
       </c>
-      <c r="H358">
+      <c r="H358" s="1">
         <v>0.8867400416544984</v>
       </c>
     </row>
@@ -7951,7 +7951,7 @@
       <c r="G362" s="1">
         <v>-4.000417301084121</v>
       </c>
-      <c r="H362">
+      <c r="H362" s="1">
         <v>-2.606818454421251</v>
       </c>
     </row>
@@ -7977,7 +7977,7 @@
       <c r="G363" s="1">
         <v>-1.912294662764338</v>
       </c>
-      <c r="H363">
+      <c r="H363" s="1">
         <v>-0.3512020892614878</v>
       </c>
     </row>
@@ -8003,7 +8003,7 @@
       <c r="G364" s="1">
         <v>-1.530350648272595</v>
       </c>
-      <c r="H364">
+      <c r="H364" s="1">
         <v>-0.139230706053731</v>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       <c r="G365" s="1">
         <v>-1.522058699987674</v>
       </c>
-      <c r="H365">
+      <c r="H365" s="1">
         <v>0.4381666504900092</v>
       </c>
     </row>
@@ -8055,7 +8055,7 @@
       <c r="G366" s="1">
         <v>-2.062432488382198</v>
       </c>
-      <c r="H366">
+      <c r="H366" s="1">
         <v>0.8421422264156312</v>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       <c r="G367" s="1">
         <v>-0.8745902031262747</v>
       </c>
-      <c r="H367">
+      <c r="H367" s="1">
         <v>1.46934270526139</v>
       </c>
     </row>
@@ -8107,7 +8107,7 @@
       <c r="G368" s="1">
         <v>-1.575954811601535</v>
       </c>
-      <c r="H368">
+      <c r="H368" s="1">
         <v>0.7591144298301369</v>
       </c>
     </row>
@@ -8133,7 +8133,7 @@
       <c r="G369" s="1">
         <v>-1.144966090798028</v>
       </c>
-      <c r="H369">
+      <c r="H369" s="1">
         <v>1.344563850095496</v>
       </c>
     </row>
@@ -8159,7 +8159,7 @@
       <c r="G370" s="1">
         <v>-0.1687945306777891</v>
       </c>
-      <c r="H370">
+      <c r="H370" s="1">
         <v>1.148256588619847</v>
       </c>
     </row>
@@ -8185,7 +8185,7 @@
       <c r="G371" s="1">
         <v>0.3108404765601874</v>
       </c>
-      <c r="H371">
+      <c r="H371" s="1">
         <v>1.27748703258986</v>
       </c>
     </row>
@@ -8211,7 +8211,7 @@
       <c r="G372" s="1">
         <v>-0.7374030849275288</v>
       </c>
-      <c r="H372">
+      <c r="H372" s="1">
         <v>0.2644607121807914</v>
       </c>
     </row>
@@ -8237,7 +8237,7 @@
       <c r="G373" s="1">
         <v>1.498579790028376</v>
       </c>
-      <c r="H373">
+      <c r="H373" s="1">
         <v>2.715975734229473</v>
       </c>
     </row>
@@ -8263,7 +8263,7 @@
       <c r="G374" s="1">
         <v>-0.8610833067820753</v>
       </c>
-      <c r="H374">
+      <c r="H374" s="1">
         <v>0.4749084948005612</v>
       </c>
     </row>
@@ -8289,7 +8289,7 @@
       <c r="G375" s="1">
         <v>0.09105692280961741</v>
       </c>
-      <c r="H375">
+      <c r="H375" s="1">
         <v>3.882701724248067</v>
       </c>
     </row>
@@ -8315,7 +8315,7 @@
       <c r="G376" s="1">
         <v>-1.094813380716308</v>
       </c>
-      <c r="H376">
+      <c r="H376" s="1">
         <v>0.5851765342471886</v>
       </c>
     </row>
@@ -8341,7 +8341,7 @@
       <c r="G377" s="1">
         <v>-0.793898663225588</v>
       </c>
-      <c r="H377">
+      <c r="H377" s="1">
         <v>0.9518238887025006</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed excel output (number format) .. now including column B!
</commit_message>
<xml_diff>
--- a/assets_output/09_logistic_regression_blocks.xlsx
+++ b/assets_output/09_logistic_regression_blocks.xlsx
@@ -49,7 +49,7 @@
     <t>rt_outcome</t>
   </si>
   <si>
-    <t>2026-06-20 12:03</t>
+    <t>2026-06-20 12:08</t>
   </si>
   <si>
     <t>2679</t>
@@ -268,9 +268,6 @@
     <t>multiple_returns</t>
   </si>
   <si>
-    <t>2026-06-20 12:04</t>
-  </si>
-  <si>
     <t>3015</t>
   </si>
   <si>
@@ -314,6 +311,9 @@
   </si>
   <si>
     <t>has_longer_term_rt</t>
+  </si>
+  <si>
+    <t>2026-06-20 12:09</t>
   </si>
   <si>
     <t>3032</t>
@@ -855,7 +855,7 @@
   <dimension ref="A1:H476"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="8" width="9.140625" style="1"/>
+    <col min="2" max="8" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -881,7 +881,7 @@
       <c r="A3" s="2">
         <v>0</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -898,7 +898,7 @@
       <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -915,7 +915,7 @@
       <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -932,7 +932,7 @@
       <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -949,7 +949,7 @@
       <c r="A7" s="2">
         <v>4</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -966,7 +966,7 @@
       <c r="A8" s="2">
         <v>5</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -983,7 +983,7 @@
       <c r="A9" s="2">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -1000,7 +1000,7 @@
       <c r="A10" s="2">
         <v>7</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -1045,7 +1045,7 @@
       <c r="A14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C14" s="1">
@@ -1071,7 +1071,7 @@
       <c r="A15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C15" s="1">
@@ -1097,7 +1097,7 @@
       <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C16" s="1">
@@ -1123,7 +1123,7 @@
       <c r="A17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C17" s="1">
@@ -1149,7 +1149,7 @@
       <c r="A18" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C18" s="1">
@@ -1175,7 +1175,7 @@
       <c r="A19" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C19" s="1">
@@ -1201,7 +1201,7 @@
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="1">
@@ -1227,7 +1227,7 @@
       <c r="A21" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C21" s="1">
@@ -1253,7 +1253,7 @@
       <c r="A22" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C22" s="1">
@@ -1279,7 +1279,7 @@
       <c r="A23" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C23" s="1">
@@ -1305,7 +1305,7 @@
       <c r="A24" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C24" s="1">
@@ -1359,7 +1359,7 @@
       <c r="A28" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C28" s="1">
@@ -1385,7 +1385,7 @@
       <c r="A29" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C29" s="1">
@@ -1411,7 +1411,7 @@
       <c r="A30" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C30" s="1">
@@ -1437,7 +1437,7 @@
       <c r="A31" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C31" s="1">
@@ -1463,7 +1463,7 @@
       <c r="A32" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C32" s="1">
@@ -1489,7 +1489,7 @@
       <c r="A33" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C33" s="1">
@@ -1515,7 +1515,7 @@
       <c r="A34" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C34" s="1">
@@ -1541,7 +1541,7 @@
       <c r="A35" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C35" s="1">
@@ -1567,7 +1567,7 @@
       <c r="A36" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C36" s="1">
@@ -1593,7 +1593,7 @@
       <c r="A37" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C37" s="1">
@@ -1619,7 +1619,7 @@
       <c r="A38" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C38" s="1">
@@ -1673,7 +1673,7 @@
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C42" s="1">
@@ -1699,7 +1699,7 @@
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C43" s="1">
@@ -1725,7 +1725,7 @@
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C44" s="1">
@@ -1751,7 +1751,7 @@
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C45" s="1">
@@ -1777,7 +1777,7 @@
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C46" s="1">
@@ -1803,7 +1803,7 @@
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C47" s="1">
@@ -1829,7 +1829,7 @@
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C48" s="1">
@@ -1855,7 +1855,7 @@
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C49" s="1">
@@ -1881,7 +1881,7 @@
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C50" s="1">
@@ -1907,7 +1907,7 @@
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C51" s="1">
@@ -1933,7 +1933,7 @@
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C52" s="1">
@@ -2663,7 +2663,7 @@
       <c r="A92" s="2">
         <v>0</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C92" s="1" t="s">
@@ -2680,7 +2680,7 @@
       <c r="A93" s="2">
         <v>1</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C93" s="1" t="s">
@@ -2697,7 +2697,7 @@
       <c r="A94" s="2">
         <v>2</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C94" s="1" t="s">
@@ -2714,7 +2714,7 @@
       <c r="A95" s="2">
         <v>3</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C95" s="1" t="s">
@@ -2731,7 +2731,7 @@
       <c r="A96" s="2">
         <v>4</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C96" s="1" t="s">
@@ -2748,7 +2748,7 @@
       <c r="A97" s="2">
         <v>5</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C97" s="1" t="s">
@@ -2765,7 +2765,7 @@
       <c r="A98" s="2">
         <v>6</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C98" s="1" t="s">
@@ -2782,7 +2782,7 @@
       <c r="A99" s="2">
         <v>7</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C99" s="1" t="s">
@@ -2827,7 +2827,7 @@
       <c r="A103" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C103" s="1">
@@ -2853,7 +2853,7 @@
       <c r="A104" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C104" s="1">
@@ -2879,7 +2879,7 @@
       <c r="A105" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C105" s="1">
@@ -2905,7 +2905,7 @@
       <c r="A106" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C106" s="1">
@@ -2931,7 +2931,7 @@
       <c r="A107" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C107" s="1">
@@ -2957,7 +2957,7 @@
       <c r="A108" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C108" s="1">
@@ -2983,7 +2983,7 @@
       <c r="A109" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C109" s="1">
@@ -3009,7 +3009,7 @@
       <c r="A110" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C110" s="1">
@@ -3035,7 +3035,7 @@
       <c r="A111" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C111" s="1">
@@ -3089,7 +3089,7 @@
       <c r="A115" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C115" s="1">
@@ -3115,7 +3115,7 @@
       <c r="A116" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C116" s="1">
@@ -3141,7 +3141,7 @@
       <c r="A117" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C117" s="1">
@@ -3167,7 +3167,7 @@
       <c r="A118" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C118" s="1">
@@ -3193,7 +3193,7 @@
       <c r="A119" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C119" s="1">
@@ -3219,7 +3219,7 @@
       <c r="A120" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C120" s="1">
@@ -3245,7 +3245,7 @@
       <c r="A121" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C121" s="1">
@@ -3271,7 +3271,7 @@
       <c r="A122" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C122" s="1">
@@ -3297,7 +3297,7 @@
       <c r="A123" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C123" s="1">
@@ -3351,7 +3351,7 @@
       <c r="A127" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C127" s="1">
@@ -3377,7 +3377,7 @@
       <c r="A128" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C128" s="1">
@@ -3403,7 +3403,7 @@
       <c r="A129" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C129" s="1">
@@ -3429,7 +3429,7 @@
       <c r="A130" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C130" s="1">
@@ -3455,7 +3455,7 @@
       <c r="A131" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C131" s="1">
@@ -3481,7 +3481,7 @@
       <c r="A132" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C132" s="1">
@@ -3507,7 +3507,7 @@
       <c r="A133" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C133" s="1">
@@ -3533,7 +3533,7 @@
       <c r="A134" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C134" s="1">
@@ -3559,7 +3559,7 @@
       <c r="A135" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C135" s="1">
@@ -4172,7 +4172,7 @@
       <c r="A169" s="2">
         <v>0</v>
       </c>
-      <c r="B169" t="s">
+      <c r="B169" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C169" s="1" t="s">
@@ -4189,7 +4189,7 @@
       <c r="A170" s="2">
         <v>1</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B170" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C170" s="1" t="s">
@@ -4199,82 +4199,82 @@
         <v>18</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="171" spans="1:7">
       <c r="A171" s="2">
         <v>2</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B171" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="D171" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="172" spans="1:7">
       <c r="A172" s="2">
         <v>3</v>
       </c>
-      <c r="B172" t="s">
+      <c r="B172" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D172" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="173" spans="1:7">
       <c r="A173" s="2">
         <v>4</v>
       </c>
-      <c r="B173" t="s">
+      <c r="B173" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D173" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E173" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" spans="1:7">
       <c r="A174" s="2">
         <v>5</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B174" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D174" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E174" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="175" spans="1:7">
       <c r="A175" s="2">
         <v>6</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B175" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C175" s="1" t="s">
@@ -4284,14 +4284,14 @@
         <v>23</v>
       </c>
       <c r="E175" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="176" spans="1:7">
       <c r="A176" s="2">
         <v>7</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B176" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C176" s="1" t="s">
@@ -4306,7 +4306,7 @@
     </row>
     <row r="178" spans="1:7">
       <c r="A178" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="179" spans="1:7">
@@ -4317,10 +4317,10 @@
         <v>35</v>
       </c>
       <c r="D179" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E179" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="E179" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="F179" s="2" t="s">
         <v>38</v>
@@ -4333,7 +4333,7 @@
       <c r="A180" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B180">
+      <c r="B180" s="1">
         <v>-4.333940926732454</v>
       </c>
       <c r="C180" s="1">
@@ -4356,7 +4356,7 @@
       <c r="A181" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B181">
+      <c r="B181" s="1">
         <v>0.5024721662958982</v>
       </c>
       <c r="C181" s="1">
@@ -4379,7 +4379,7 @@
       <c r="A182" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B182">
+      <c r="B182" s="1">
         <v>0.7840184968228269</v>
       </c>
       <c r="C182" s="1">
@@ -4402,7 +4402,7 @@
       <c r="A183" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B183">
+      <c r="B183" s="1">
         <v>0.3872625266993386</v>
       </c>
       <c r="C183" s="1">
@@ -4425,7 +4425,7 @@
       <c r="A184" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B184">
+      <c r="B184" s="1">
         <v>1.895252685444775</v>
       </c>
       <c r="C184" s="1">
@@ -4448,7 +4448,7 @@
       <c r="A185" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B185">
+      <c r="B185" s="1">
         <v>0.5274721624755884</v>
       </c>
       <c r="C185" s="1">
@@ -4471,7 +4471,7 @@
       <c r="A186" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B186">
+      <c r="B186" s="1">
         <v>0.7722157720370918</v>
       </c>
       <c r="C186" s="1">
@@ -4492,7 +4492,7 @@
     </row>
     <row r="188" spans="1:7">
       <c r="A188" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="189" spans="1:7">
@@ -4516,7 +4516,7 @@
       <c r="A190" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B190">
+      <c r="B190" s="1">
         <v>3.403877632060557E-100</v>
       </c>
       <c r="C190" s="1" t="s">
@@ -4536,7 +4536,7 @@
       <c r="A191" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B191">
+      <c r="B191" s="1">
         <v>0.0002162299178150398</v>
       </c>
       <c r="C191" s="1" t="s">
@@ -4556,7 +4556,7 @@
       <c r="A192" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B192">
+      <c r="B192" s="1">
         <v>3.877645465391263E-08</v>
       </c>
       <c r="C192" s="1" t="s">
@@ -4576,7 +4576,7 @@
       <c r="A193" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B193">
+      <c r="B193" s="1">
         <v>0.004006522046895985</v>
       </c>
       <c r="C193" s="1" t="s">
@@ -4596,7 +4596,7 @@
       <c r="A194" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B194">
+      <c r="B194" s="1">
         <v>0.0001671667483768753</v>
       </c>
       <c r="C194" s="1" t="s">
@@ -4616,7 +4616,7 @@
       <c r="A195" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B195">
+      <c r="B195" s="1">
         <v>0.01872462001917282</v>
       </c>
       <c r="C195" s="1" t="s">
@@ -4636,7 +4636,7 @@
       <c r="A196" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B196">
+      <c r="B196" s="1">
         <v>5.644264481205005E-23</v>
       </c>
       <c r="C196" s="1" t="s">
@@ -4654,7 +4654,7 @@
     </row>
     <row r="198" spans="1:6">
       <c r="A198" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="199" spans="1:6">
@@ -4675,7 +4675,7 @@
       <c r="A200" s="2">
         <v>0</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B200" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C200" s="1" t="s">
@@ -4692,11 +4692,11 @@
       <c r="A201" s="2">
         <v>1</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B201" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C201" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D201" s="1" t="s">
         <v>18</v>
@@ -4709,11 +4709,11 @@
       <c r="A202" s="2">
         <v>2</v>
       </c>
-      <c r="B202" t="s">
+      <c r="B202" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="D202" s="1" t="s">
         <v>19</v>
@@ -4726,7 +4726,7 @@
       <c r="A203" s="2">
         <v>3</v>
       </c>
-      <c r="B203" t="s">
+      <c r="B203" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C203" s="1" t="s">
@@ -4743,11 +4743,11 @@
       <c r="A204" s="2">
         <v>4</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B204" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D204" s="1" t="s">
         <v>21</v>
@@ -4760,7 +4760,7 @@
       <c r="A205" s="2">
         <v>5</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B205" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C205" s="1" t="s">
@@ -4777,7 +4777,7 @@
       <c r="A206" s="2">
         <v>6</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B206" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C206" s="1" t="s">
@@ -4794,7 +4794,7 @@
       <c r="A207" s="2">
         <v>7</v>
       </c>
-      <c r="B207" t="s">
+      <c r="B207" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C207" s="1" t="s">
@@ -4820,10 +4820,10 @@
         <v>35</v>
       </c>
       <c r="D210" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E210" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="E210" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="F210" s="2" t="s">
         <v>38</v>
@@ -4836,7 +4836,7 @@
       <c r="A211" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B211">
+      <c r="B211" s="1">
         <v>-1.147198797506423</v>
       </c>
       <c r="C211" s="1">
@@ -4859,7 +4859,7 @@
       <c r="A212" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B212">
+      <c r="B212" s="1">
         <v>-0.5288436847696434</v>
       </c>
       <c r="C212" s="1">
@@ -4882,7 +4882,7 @@
       <c r="A213" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B213">
+      <c r="B213" s="1">
         <v>-1.11558867186674</v>
       </c>
       <c r="C213" s="1">
@@ -4905,7 +4905,7 @@
       <c r="A214" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B214">
+      <c r="B214" s="1">
         <v>-0.5562121563176856</v>
       </c>
       <c r="C214" s="1">
@@ -4928,7 +4928,7 @@
       <c r="A215" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B215">
+      <c r="B215" s="1">
         <v>-0.7739634004747185</v>
       </c>
       <c r="C215" s="1">
@@ -4951,7 +4951,7 @@
       <c r="A216" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B216">
+      <c r="B216" s="1">
         <v>-1.207732428258562</v>
       </c>
       <c r="C216" s="1">
@@ -4974,7 +4974,7 @@
       <c r="A217" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B217">
+      <c r="B217" s="1">
         <v>0.4898034909014749</v>
       </c>
       <c r="C217" s="1">
@@ -5019,7 +5019,7 @@
       <c r="A221" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B221">
+      <c r="B221" s="1">
         <v>7.285949456051732E-54</v>
       </c>
       <c r="C221" s="1" t="s">
@@ -5039,7 +5039,7 @@
       <c r="A222" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B222">
+      <c r="B222" s="1">
         <v>7.537727985363454E-07</v>
       </c>
       <c r="C222" s="1" t="s">
@@ -5059,7 +5059,7 @@
       <c r="A223" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B223">
+      <c r="B223" s="1">
         <v>3.024980425802322E-05</v>
       </c>
       <c r="C223" s="1" t="s">
@@ -5079,7 +5079,7 @@
       <c r="A224" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B224">
+      <c r="B224" s="1">
         <v>0.2824771975296116</v>
       </c>
       <c r="D224" s="1">
@@ -5096,7 +5096,7 @@
       <c r="A225" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B225">
+      <c r="B225" s="1">
         <v>4.231429130550076E-06</v>
       </c>
       <c r="C225" s="1" t="s">
@@ -5116,7 +5116,7 @@
       <c r="A226" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B226">
+      <c r="B226" s="1">
         <v>0.005169534398375955</v>
       </c>
       <c r="C226" s="1" t="s">
@@ -5136,7 +5136,7 @@
       <c r="A227" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B227">
+      <c r="B227" s="1">
         <v>6.031114858474766E-12</v>
       </c>
       <c r="C227" s="1" t="s">
@@ -5175,7 +5175,7 @@
       <c r="A231" s="2">
         <v>0</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B231" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C231" s="1" t="s">
@@ -5192,7 +5192,7 @@
       <c r="A232" s="2">
         <v>1</v>
       </c>
-      <c r="B232" t="s">
+      <c r="B232" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C232" s="1" t="s">
@@ -5209,11 +5209,11 @@
       <c r="A233" s="2">
         <v>2</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B233" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="D233" s="1" t="s">
         <v>19</v>
@@ -5226,7 +5226,7 @@
       <c r="A234" s="2">
         <v>3</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B234" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C234" s="1" t="s">
@@ -5243,7 +5243,7 @@
       <c r="A235" s="2">
         <v>4</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B235" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C235" s="1" t="s">
@@ -5260,7 +5260,7 @@
       <c r="A236" s="2">
         <v>5</v>
       </c>
-      <c r="B236" t="s">
+      <c r="B236" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C236" s="1" t="s">
@@ -5277,7 +5277,7 @@
       <c r="A237" s="2">
         <v>6</v>
       </c>
-      <c r="B237" t="s">
+      <c r="B237" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C237" s="1" t="s">
@@ -5294,7 +5294,7 @@
       <c r="A238" s="2">
         <v>7</v>
       </c>
-      <c r="B238" t="s">
+      <c r="B238" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C238" s="1" t="s">
@@ -5320,10 +5320,10 @@
         <v>35</v>
       </c>
       <c r="D241" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E241" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="E241" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="F241" s="2" t="s">
         <v>38</v>
@@ -5336,7 +5336,7 @@
       <c r="A242" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B242">
+      <c r="B242" s="1">
         <v>-5.389729049222971</v>
       </c>
       <c r="C242" s="1">
@@ -5359,7 +5359,7 @@
       <c r="A243" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B243">
+      <c r="B243" s="1">
         <v>2.475108324951747</v>
       </c>
       <c r="C243" s="1">
@@ -5382,7 +5382,7 @@
       <c r="A244" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B244">
+      <c r="B244" s="1">
         <v>2.648706171830171</v>
       </c>
       <c r="C244" s="1">
@@ -5405,7 +5405,7 @@
       <c r="A245" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B245">
+      <c r="B245" s="1">
         <v>1.172146522488462</v>
       </c>
       <c r="C245" s="1">
@@ -5450,7 +5450,7 @@
       <c r="A249" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B249">
+      <c r="B249" s="1">
         <v>3.222904910656649E-17</v>
       </c>
       <c r="C249" s="1" t="s">
@@ -5470,7 +5470,7 @@
       <c r="A250" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B250">
+      <c r="B250" s="1">
         <v>0.0004389868297785795</v>
       </c>
       <c r="C250" s="1" t="s">
@@ -5490,7 +5490,7 @@
       <c r="A251" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B251">
+      <c r="B251" s="1">
         <v>0.03919733536927187</v>
       </c>
       <c r="C251" s="1" t="s">
@@ -5510,7 +5510,7 @@
       <c r="A252" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B252">
+      <c r="B252" s="1">
         <v>3.086842961632247E-05</v>
       </c>
       <c r="C252" s="1" t="s">
@@ -5549,7 +5549,7 @@
       <c r="A256" s="2">
         <v>0</v>
       </c>
-      <c r="B256" t="s">
+      <c r="B256" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C256" s="1" t="s">
@@ -5566,7 +5566,7 @@
       <c r="A257" s="2">
         <v>1</v>
       </c>
-      <c r="B257" t="s">
+      <c r="B257" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C257" s="1" t="s">
@@ -5583,11 +5583,11 @@
       <c r="A258" s="2">
         <v>2</v>
       </c>
-      <c r="B258" t="s">
+      <c r="B258" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="D258" s="1" t="s">
         <v>19</v>
@@ -5600,7 +5600,7 @@
       <c r="A259" s="2">
         <v>3</v>
       </c>
-      <c r="B259" t="s">
+      <c r="B259" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C259" s="1" t="s">
@@ -5617,7 +5617,7 @@
       <c r="A260" s="2">
         <v>4</v>
       </c>
-      <c r="B260" t="s">
+      <c r="B260" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C260" s="1" t="s">
@@ -5634,7 +5634,7 @@
       <c r="A261" s="2">
         <v>5</v>
       </c>
-      <c r="B261" t="s">
+      <c r="B261" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C261" s="1" t="s">
@@ -5651,7 +5651,7 @@
       <c r="A262" s="2">
         <v>6</v>
       </c>
-      <c r="B262" t="s">
+      <c r="B262" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C262" s="1" t="s">
@@ -5668,7 +5668,7 @@
       <c r="A263" s="2">
         <v>7</v>
       </c>
-      <c r="B263" t="s">
+      <c r="B263" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C263" s="1" t="s">
@@ -5713,7 +5713,7 @@
       <c r="A267" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B267" t="s">
+      <c r="B267" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C267" s="1">
@@ -5739,7 +5739,7 @@
       <c r="A268" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B268" t="s">
+      <c r="B268" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C268" s="1">
@@ -5765,7 +5765,7 @@
       <c r="A269" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B269" t="s">
+      <c r="B269" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C269" s="1">
@@ -5791,7 +5791,7 @@
       <c r="A270" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B270" t="s">
+      <c r="B270" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C270" s="1">
@@ -5817,7 +5817,7 @@
       <c r="A271" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B271" t="s">
+      <c r="B271" s="1" t="s">
         <v>141</v>
       </c>
       <c r="C271" s="1">
@@ -5843,7 +5843,7 @@
       <c r="A272" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B272" t="s">
+      <c r="B272" s="1" t="s">
         <v>142</v>
       </c>
       <c r="C272" s="1">
@@ -5869,7 +5869,7 @@
       <c r="A273" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B273" t="s">
+      <c r="B273" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C273" s="1">
@@ -5895,7 +5895,7 @@
       <c r="A274" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B274" t="s">
+      <c r="B274" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C274" s="1">
@@ -5921,7 +5921,7 @@
       <c r="A275" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B275" t="s">
+      <c r="B275" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C275" s="1">
@@ -5947,7 +5947,7 @@
       <c r="A276" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B276" t="s">
+      <c r="B276" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C276" s="1">
@@ -5973,7 +5973,7 @@
       <c r="A277" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B277" t="s">
+      <c r="B277" s="1" t="s">
         <v>143</v>
       </c>
       <c r="C277" s="1">
@@ -5999,7 +5999,7 @@
       <c r="A278" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B278" t="s">
+      <c r="B278" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C278" s="1">
@@ -6025,7 +6025,7 @@
       <c r="A279" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B279" t="s">
+      <c r="B279" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C279" s="1">
@@ -6051,7 +6051,7 @@
       <c r="A280" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B280" t="s">
+      <c r="B280" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C280" s="1">
@@ -6077,7 +6077,7 @@
       <c r="A281" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B281" t="s">
+      <c r="B281" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C281" s="1">
@@ -6103,7 +6103,7 @@
       <c r="A282" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B282" t="s">
+      <c r="B282" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C282" s="1">
@@ -6157,7 +6157,7 @@
       <c r="A286" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B286" t="s">
+      <c r="B286" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C286" s="1">
@@ -6183,7 +6183,7 @@
       <c r="A287" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B287" t="s">
+      <c r="B287" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C287" s="1">
@@ -6209,7 +6209,7 @@
       <c r="A288" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B288" t="s">
+      <c r="B288" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C288" s="1">
@@ -6235,7 +6235,7 @@
       <c r="A289" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B289" t="s">
+      <c r="B289" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C289" s="1">
@@ -6261,7 +6261,7 @@
       <c r="A290" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B290" t="s">
+      <c r="B290" s="1" t="s">
         <v>141</v>
       </c>
       <c r="C290" s="1">
@@ -6287,7 +6287,7 @@
       <c r="A291" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B291" t="s">
+      <c r="B291" s="1" t="s">
         <v>142</v>
       </c>
       <c r="C291" s="1">
@@ -6313,7 +6313,7 @@
       <c r="A292" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B292" t="s">
+      <c r="B292" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C292" s="1">
@@ -6339,7 +6339,7 @@
       <c r="A293" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B293" t="s">
+      <c r="B293" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C293" s="1">
@@ -6365,7 +6365,7 @@
       <c r="A294" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B294" t="s">
+      <c r="B294" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C294" s="1">
@@ -6391,7 +6391,7 @@
       <c r="A295" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B295" t="s">
+      <c r="B295" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C295" s="1">
@@ -6417,7 +6417,7 @@
       <c r="A296" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B296" t="s">
+      <c r="B296" s="1" t="s">
         <v>143</v>
       </c>
       <c r="C296" s="1">
@@ -6443,7 +6443,7 @@
       <c r="A297" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B297" t="s">
+      <c r="B297" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C297" s="1">
@@ -6469,7 +6469,7 @@
       <c r="A298" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B298" t="s">
+      <c r="B298" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C298" s="1">
@@ -6495,7 +6495,7 @@
       <c r="A299" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B299" t="s">
+      <c r="B299" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C299" s="1">
@@ -6521,7 +6521,7 @@
       <c r="A300" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B300" t="s">
+      <c r="B300" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C300" s="1">
@@ -6547,7 +6547,7 @@
       <c r="A301" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B301" t="s">
+      <c r="B301" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C301" s="1">
@@ -6601,7 +6601,7 @@
       <c r="A305" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B305" t="s">
+      <c r="B305" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C305" s="1">
@@ -6627,7 +6627,7 @@
       <c r="A306" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B306" t="s">
+      <c r="B306" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C306" s="1">
@@ -6653,7 +6653,7 @@
       <c r="A307" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B307" t="s">
+      <c r="B307" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C307" s="1">
@@ -6679,7 +6679,7 @@
       <c r="A308" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B308" t="s">
+      <c r="B308" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C308" s="1">
@@ -6705,7 +6705,7 @@
       <c r="A309" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B309" t="s">
+      <c r="B309" s="1" t="s">
         <v>141</v>
       </c>
       <c r="C309" s="1">
@@ -6731,7 +6731,7 @@
       <c r="A310" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B310" t="s">
+      <c r="B310" s="1" t="s">
         <v>142</v>
       </c>
       <c r="C310" s="1">
@@ -6757,7 +6757,7 @@
       <c r="A311" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B311" t="s">
+      <c r="B311" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C311" s="1">
@@ -6783,7 +6783,7 @@
       <c r="A312" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B312" t="s">
+      <c r="B312" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C312" s="1">
@@ -6809,7 +6809,7 @@
       <c r="A313" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B313" t="s">
+      <c r="B313" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C313" s="1">
@@ -6835,7 +6835,7 @@
       <c r="A314" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B314" t="s">
+      <c r="B314" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C314" s="1">
@@ -6861,7 +6861,7 @@
       <c r="A315" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B315" t="s">
+      <c r="B315" s="1" t="s">
         <v>143</v>
       </c>
       <c r="C315" s="1">
@@ -6887,7 +6887,7 @@
       <c r="A316" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B316" t="s">
+      <c r="B316" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C316" s="1">
@@ -6913,7 +6913,7 @@
       <c r="A317" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B317" t="s">
+      <c r="B317" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C317" s="1">
@@ -6939,7 +6939,7 @@
       <c r="A318" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B318" t="s">
+      <c r="B318" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C318" s="1">
@@ -6965,7 +6965,7 @@
       <c r="A319" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B319" t="s">
+      <c r="B319" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C319" s="1">
@@ -6991,7 +6991,7 @@
       <c r="A320" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B320" t="s">
+      <c r="B320" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C320" s="1">
@@ -7045,7 +7045,7 @@
       <c r="A324" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B324" t="s">
+      <c r="B324" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C324" s="1">
@@ -7071,7 +7071,7 @@
       <c r="A325" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B325" t="s">
+      <c r="B325" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C325" s="1">
@@ -7097,7 +7097,7 @@
       <c r="A326" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B326" t="s">
+      <c r="B326" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C326" s="1">
@@ -7123,7 +7123,7 @@
       <c r="A327" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B327" t="s">
+      <c r="B327" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C327" s="1">
@@ -7149,7 +7149,7 @@
       <c r="A328" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B328" t="s">
+      <c r="B328" s="1" t="s">
         <v>141</v>
       </c>
       <c r="C328" s="1">
@@ -7175,7 +7175,7 @@
       <c r="A329" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B329" t="s">
+      <c r="B329" s="1" t="s">
         <v>142</v>
       </c>
       <c r="C329" s="1">
@@ -7201,7 +7201,7 @@
       <c r="A330" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B330" t="s">
+      <c r="B330" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C330" s="1">
@@ -7227,7 +7227,7 @@
       <c r="A331" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B331" t="s">
+      <c r="B331" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C331" s="1">
@@ -7253,7 +7253,7 @@
       <c r="A332" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B332" t="s">
+      <c r="B332" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C332" s="1">
@@ -7279,7 +7279,7 @@
       <c r="A333" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B333" t="s">
+      <c r="B333" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C333" s="1">
@@ -7305,7 +7305,7 @@
       <c r="A334" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B334" t="s">
+      <c r="B334" s="1" t="s">
         <v>143</v>
       </c>
       <c r="C334" s="1">
@@ -7331,7 +7331,7 @@
       <c r="A335" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B335" t="s">
+      <c r="B335" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C335" s="1">
@@ -7357,7 +7357,7 @@
       <c r="A336" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B336" t="s">
+      <c r="B336" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C336" s="1">
@@ -7383,7 +7383,7 @@
       <c r="A337" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B337" t="s">
+      <c r="B337" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C337" s="1">
@@ -7409,7 +7409,7 @@
       <c r="A338" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B338" t="s">
+      <c r="B338" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C338" s="1">
@@ -7435,7 +7435,7 @@
       <c r="A339" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B339" t="s">
+      <c r="B339" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C339" s="1">
@@ -7489,7 +7489,7 @@
       <c r="A343" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B343" t="s">
+      <c r="B343" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C343" s="1">
@@ -7515,7 +7515,7 @@
       <c r="A344" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B344" t="s">
+      <c r="B344" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C344" s="1">
@@ -7541,7 +7541,7 @@
       <c r="A345" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B345" t="s">
+      <c r="B345" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C345" s="1">
@@ -7567,7 +7567,7 @@
       <c r="A346" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B346" t="s">
+      <c r="B346" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C346" s="1">
@@ -7593,7 +7593,7 @@
       <c r="A347" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B347" t="s">
+      <c r="B347" s="1" t="s">
         <v>141</v>
       </c>
       <c r="C347" s="1">
@@ -7619,7 +7619,7 @@
       <c r="A348" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B348" t="s">
+      <c r="B348" s="1" t="s">
         <v>142</v>
       </c>
       <c r="C348" s="1">
@@ -7645,7 +7645,7 @@
       <c r="A349" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B349" t="s">
+      <c r="B349" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C349" s="1">
@@ -7671,7 +7671,7 @@
       <c r="A350" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B350" t="s">
+      <c r="B350" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C350" s="1">
@@ -7697,7 +7697,7 @@
       <c r="A351" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B351" t="s">
+      <c r="B351" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C351" s="1">
@@ -7723,7 +7723,7 @@
       <c r="A352" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B352" t="s">
+      <c r="B352" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C352" s="1">
@@ -7749,7 +7749,7 @@
       <c r="A353" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B353" t="s">
+      <c r="B353" s="1" t="s">
         <v>143</v>
       </c>
       <c r="C353" s="1">
@@ -7775,7 +7775,7 @@
       <c r="A354" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B354" t="s">
+      <c r="B354" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C354" s="1">
@@ -7801,7 +7801,7 @@
       <c r="A355" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B355" t="s">
+      <c r="B355" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C355" s="1">
@@ -7827,7 +7827,7 @@
       <c r="A356" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B356" t="s">
+      <c r="B356" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C356" s="1">
@@ -7853,7 +7853,7 @@
       <c r="A357" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B357" t="s">
+      <c r="B357" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C357" s="1">
@@ -7879,7 +7879,7 @@
       <c r="A358" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B358" t="s">
+      <c r="B358" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C358" s="1">
@@ -7933,7 +7933,7 @@
       <c r="A362" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B362" t="s">
+      <c r="B362" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C362" s="1">
@@ -7959,7 +7959,7 @@
       <c r="A363" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B363" t="s">
+      <c r="B363" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C363" s="1">
@@ -7985,7 +7985,7 @@
       <c r="A364" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B364" t="s">
+      <c r="B364" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C364" s="1">
@@ -8011,7 +8011,7 @@
       <c r="A365" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B365" t="s">
+      <c r="B365" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C365" s="1">
@@ -8037,7 +8037,7 @@
       <c r="A366" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B366" t="s">
+      <c r="B366" s="1" t="s">
         <v>141</v>
       </c>
       <c r="C366" s="1">
@@ -8063,7 +8063,7 @@
       <c r="A367" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B367" t="s">
+      <c r="B367" s="1" t="s">
         <v>142</v>
       </c>
       <c r="C367" s="1">
@@ -8089,7 +8089,7 @@
       <c r="A368" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B368" t="s">
+      <c r="B368" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C368" s="1">
@@ -8115,7 +8115,7 @@
       <c r="A369" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B369" t="s">
+      <c r="B369" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C369" s="1">
@@ -8141,7 +8141,7 @@
       <c r="A370" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B370" t="s">
+      <c r="B370" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C370" s="1">
@@ -8167,7 +8167,7 @@
       <c r="A371" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B371" t="s">
+      <c r="B371" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C371" s="1">
@@ -8193,7 +8193,7 @@
       <c r="A372" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B372" t="s">
+      <c r="B372" s="1" t="s">
         <v>143</v>
       </c>
       <c r="C372" s="1">
@@ -8219,7 +8219,7 @@
       <c r="A373" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B373" t="s">
+      <c r="B373" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C373" s="1">
@@ -8245,7 +8245,7 @@
       <c r="A374" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B374" t="s">
+      <c r="B374" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C374" s="1">
@@ -8271,7 +8271,7 @@
       <c r="A375" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B375" t="s">
+      <c r="B375" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C375" s="1">
@@ -8297,7 +8297,7 @@
       <c r="A376" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B376" t="s">
+      <c r="B376" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C376" s="1">
@@ -8323,7 +8323,7 @@
       <c r="A377" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B377" t="s">
+      <c r="B377" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C377" s="1">

</xml_diff>

<commit_message>
Fixed category names in MNLogit excel export
</commit_message>
<xml_diff>
--- a/assets_output/09_logistic_regression_blocks.xlsx
+++ b/assets_output/09_logistic_regression_blocks.xlsx
@@ -49,7 +49,7 @@
     <t>rt_outcome</t>
   </si>
   <si>
-    <t>2026-06-20 12:08</t>
+    <t>2026-06-20 12:49</t>
   </si>
   <si>
     <t>2679</t>
@@ -115,7 +115,7 @@
     <t>MNLogit: 'Route outcomes after 3.08 years', table 1</t>
   </si>
   <si>
-    <t>rt_outcome = 0</t>
+    <t>rt_outcome=Insecure outcome</t>
   </si>
   <si>
     <t>Coef.</t>
@@ -172,13 +172,13 @@
     <t>MNLogit: 'Route outcomes after 3.08 years', table 2</t>
   </si>
   <si>
-    <t>rt_outcome = 1</t>
+    <t>rt_outcome=Returned to homelessness</t>
   </si>
   <si>
     <t>MNLogit: 'Route outcomes after 3.08 years', table 3</t>
   </si>
   <si>
-    <t>rt_outcome = 2</t>
+    <t>rt_outcome=Died</t>
   </si>
   <si>
     <t>MNLogit: 'Route outcomes after 3.08 years', odds ratios</t>
@@ -241,19 +241,19 @@
     <t>MNLogit: 'Outcomes 3.08 years after a person's first route started', table 1</t>
   </si>
   <si>
-    <t>cli_outcome = 0</t>
+    <t>cli_outcome=Insecure outcome</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes 3.08 years after a person's first route started', table 2</t>
   </si>
   <si>
-    <t>cli_outcome = 1</t>
+    <t>cli_outcome=Returned to homelessness</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes 3.08 years after a person's first route started', table 3</t>
   </si>
   <si>
-    <t>cli_outcome = 2</t>
+    <t>cli_outcome=Died</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes 3.08 years after a person's first route started', odds ratios</t>
@@ -313,9 +313,6 @@
     <t>has_longer_term_rt</t>
   </si>
   <si>
-    <t>2026-06-20 12:09</t>
-  </si>
-  <si>
     <t>3032</t>
   </si>
   <si>
@@ -403,6 +400,9 @@
     <t>pl_outcome</t>
   </si>
   <si>
+    <t>2026-06-20 12:50</t>
+  </si>
+  <si>
     <t>5016</t>
   </si>
   <si>
@@ -433,7 +433,7 @@
     <t>MNLogit: 'Outcomes from individual placements', table 1</t>
   </si>
   <si>
-    <t>pl_outcome = 0</t>
+    <t>pl_outcome=Internal move: forwards</t>
   </si>
   <si>
     <t>ethnicity_grouped_Black</t>
@@ -451,31 +451,31 @@
     <t>MNLogit: 'Outcomes from individual placements', table 2</t>
   </si>
   <si>
-    <t>pl_outcome = 1</t>
+    <t>pl_outcome=Internal move: sideways</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes from individual placements', table 3</t>
   </si>
   <si>
-    <t>pl_outcome = 2</t>
+    <t>pl_outcome=Internal move: backwards</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes from individual placements', table 4</t>
   </si>
   <si>
-    <t>pl_outcome = 3</t>
+    <t>pl_outcome=Returned to homelessness</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes from individual placements', table 5</t>
   </si>
   <si>
-    <t>pl_outcome = 4</t>
+    <t>pl_outcome=Insecure outcome (external)</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes from individual placements', table 6</t>
   </si>
   <si>
-    <t>pl_outcome = 5</t>
+    <t>pl_outcome=Died</t>
   </si>
   <si>
     <t>MNLogit: 'Outcomes from individual placements', odds ratios</t>
@@ -4702,7 +4702,7 @@
         <v>18</v>
       </c>
       <c r="E201" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="202" spans="1:6">
@@ -4713,13 +4713,13 @@
         <v>3</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>99</v>
+        <v>11</v>
       </c>
       <c r="D202" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E202" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="203" spans="1:6">
@@ -4730,13 +4730,13 @@
         <v>4</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D203" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E203" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="204" spans="1:6">
@@ -4753,7 +4753,7 @@
         <v>21</v>
       </c>
       <c r="E204" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="205" spans="1:6">
@@ -4764,13 +4764,13 @@
         <v>6</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D205" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E205" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="206" spans="1:6">
@@ -4787,7 +4787,7 @@
         <v>23</v>
       </c>
       <c r="E206" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="207" spans="1:6">
@@ -4798,7 +4798,7 @@
         <v>8</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D207" s="1" t="s">
         <v>24</v>
@@ -4809,7 +4809,7 @@
     </row>
     <row r="209" spans="1:7">
       <c r="A209" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="210" spans="1:7">
@@ -4880,7 +4880,7 @@
     </row>
     <row r="213" spans="1:7">
       <c r="A213" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B213" s="1">
         <v>-1.11558867186674</v>
@@ -4995,7 +4995,7 @@
     </row>
     <row r="219" spans="1:7">
       <c r="A219" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="220" spans="1:7">
@@ -5077,7 +5077,7 @@
     </row>
     <row r="224" spans="1:7">
       <c r="A224" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B224" s="1">
         <v>0.2824771975296116</v>
@@ -5154,7 +5154,7 @@
     </row>
     <row r="229" spans="1:6">
       <c r="A229" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="230" spans="1:6">
@@ -5196,13 +5196,13 @@
         <v>2</v>
       </c>
       <c r="C232" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D232" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E232" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="233" spans="1:6">
@@ -5213,13 +5213,13 @@
         <v>3</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>99</v>
+        <v>11</v>
       </c>
       <c r="D233" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E233" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="234" spans="1:6">
@@ -5230,13 +5230,13 @@
         <v>4</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D234" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E234" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="235" spans="1:6">
@@ -5247,13 +5247,13 @@
         <v>5</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D235" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E235" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="236" spans="1:6">
@@ -5264,13 +5264,13 @@
         <v>6</v>
       </c>
       <c r="C236" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D236" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E236" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="237" spans="1:6">
@@ -5287,7 +5287,7 @@
         <v>23</v>
       </c>
       <c r="E237" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="238" spans="1:6">
@@ -5309,7 +5309,7 @@
     </row>
     <row r="240" spans="1:6">
       <c r="A240" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="241" spans="1:7">
@@ -5357,7 +5357,7 @@
     </row>
     <row r="243" spans="1:7">
       <c r="A243" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B243" s="1">
         <v>2.475108324951747</v>
@@ -5403,7 +5403,7 @@
     </row>
     <row r="245" spans="1:7">
       <c r="A245" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B245" s="1">
         <v>1.172146522488462</v>
@@ -5426,7 +5426,7 @@
     </row>
     <row r="247" spans="1:7">
       <c r="A247" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="248" spans="1:7">
@@ -5468,7 +5468,7 @@
     </row>
     <row r="250" spans="1:7">
       <c r="A250" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B250" s="1">
         <v>0.0004389868297785795</v>
@@ -5488,7 +5488,7 @@
     </row>
     <row r="251" spans="1:7">
       <c r="A251" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B251" s="1">
         <v>0.03919733536927187</v>
@@ -5528,7 +5528,7 @@
     </row>
     <row r="254" spans="1:7">
       <c r="A254" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="255" spans="1:7">
@@ -5570,7 +5570,7 @@
         <v>2</v>
       </c>
       <c r="C257" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D257" s="1" t="s">
         <v>18</v>
@@ -5587,7 +5587,7 @@
         <v>3</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="D258" s="1" t="s">
         <v>19</v>
@@ -6075,10 +6075,10 @@
     </row>
     <row r="281" spans="1:8">
       <c r="A281" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C281" s="1">
         <v>0.132899369457811</v>
@@ -6519,10 +6519,10 @@
     </row>
     <row r="300" spans="1:8">
       <c r="A300" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C300" s="1">
         <v>0.1221421410218785</v>
@@ -6963,10 +6963,10 @@
     </row>
     <row r="319" spans="1:8">
       <c r="A319" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C319" s="1">
         <v>0.2552177671192801</v>
@@ -7407,10 +7407,10 @@
     </row>
     <row r="338" spans="1:8">
       <c r="A338" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B338" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C338" s="1">
         <v>0.4220748693433146</v>
@@ -7851,10 +7851,10 @@
     </row>
     <row r="357" spans="1:8">
       <c r="A357" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C357" s="1">
         <v>0.1773128236392056</v>
@@ -8295,10 +8295,10 @@
     </row>
     <row r="376" spans="1:8">
       <c r="A376" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C376" s="1">
         <v>-0.2548184232345599</v>
@@ -8561,7 +8561,7 @@
     <row r="391" spans="1:7">
       <c r="A391" s="2"/>
       <c r="B391" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C391" s="1">
         <v>0.3243426031463325</v>
@@ -8878,7 +8878,7 @@
     <row r="407" spans="1:7">
       <c r="A407" s="2"/>
       <c r="B407" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C407" s="1">
         <v>0.4183881489014909</v>
@@ -9192,7 +9192,7 @@
     <row r="423" spans="1:7">
       <c r="A423" s="2"/>
       <c r="B423" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C423" s="1">
         <v>0.1147765647959176</v>
@@ -9500,7 +9500,7 @@
     <row r="439" spans="1:7">
       <c r="A439" s="2"/>
       <c r="B439" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C439" s="1">
         <v>0.009820048795527999</v>
@@ -9817,7 +9817,7 @@
     <row r="455" spans="1:7">
       <c r="A455" s="2"/>
       <c r="B455" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C455" s="1">
         <v>0.3090265089901769</v>
@@ -10125,7 +10125,7 @@
     <row r="471" spans="1:7">
       <c r="A471" s="2"/>
       <c r="B471" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C471" s="1">
         <v>0.552131630609431</v>

</xml_diff>

<commit_message>
Added individual placement outcomes MNLogit with two different reference categories.
</commit_message>
<xml_diff>
--- a/assets_output/09_logistic_regression_blocks.xlsx
+++ b/assets_output/09_logistic_regression_blocks.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1325" uniqueCount="179">
   <si>
     <t>MNLogit: 'Route outcomes after 3.08 years', table 0</t>
   </si>
@@ -49,7 +49,7 @@
     <t>rt_outcome</t>
   </si>
   <si>
-    <t>2026-06-20 12:49</t>
+    <t>2026-06-21 13:14</t>
   </si>
   <si>
     <t>2679</t>
@@ -208,6 +208,9 @@
     <t>cli_outcome</t>
   </si>
   <si>
+    <t>2026-06-21 13:15</t>
+  </si>
+  <si>
     <t>2014</t>
   </si>
   <si>
@@ -394,15 +397,12 @@
     <t>Logit: 'Returns within 2 years after moving to independent accommodation', odds ratios</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', table 0</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', table 0</t>
   </si>
   <si>
     <t>pl_outcome</t>
   </si>
   <si>
-    <t>2026-06-20 12:50</t>
-  </si>
-  <si>
     <t>5016</t>
   </si>
   <si>
@@ -430,7 +430,7 @@
     <t>1.6272e-190</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', table 1</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', table 1</t>
   </si>
   <si>
     <t>pl_outcome=Internal move: forwards</t>
@@ -448,37 +448,37 @@
     <t>mental_health</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', table 2</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', table 2</t>
   </si>
   <si>
     <t>pl_outcome=Internal move: sideways</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', table 3</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', table 3</t>
   </si>
   <si>
     <t>pl_outcome=Internal move: backwards</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', table 4</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', table 4</t>
   </si>
   <si>
     <t>pl_outcome=Returned to homelessness</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', table 5</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', table 5</t>
   </si>
   <si>
     <t>pl_outcome=Insecure outcome (external)</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', table 6</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', table 6</t>
   </si>
   <si>
     <t>pl_outcome=Died</t>
   </si>
   <si>
-    <t>MNLogit: 'Outcomes from individual placements', odds ratios</t>
+    <t>MNLogit: 'Outcomes from individual placements (vs independent accommodation)', odds ratios</t>
   </si>
   <si>
     <t>Internal move: forwards</t>
@@ -491,6 +491,66 @@
   </si>
   <si>
     <t>Insecure outcome (external)</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 0</t>
+  </si>
+  <si>
+    <t>2026-06-21 13:16</t>
+  </si>
+  <si>
+    <t>5191</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>5113</t>
+  </si>
+  <si>
+    <t>0.065</t>
+  </si>
+  <si>
+    <t>17455.0005</t>
+  </si>
+  <si>
+    <t>17966.2657</t>
+  </si>
+  <si>
+    <t>-8649.5</t>
+  </si>
+  <si>
+    <t>-9247.8</t>
+  </si>
+  <si>
+    <t>2.4311e-203</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 1</t>
+  </si>
+  <si>
+    <t>pl_outcome=Independent accommodation</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 2</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 3</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 4</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 5</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 6</t>
+  </si>
+  <si>
+    <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', odds ratios</t>
+  </si>
+  <si>
+    <t>Independent accommodation</t>
   </si>
 </sst>
 </file>
@@ -852,7 +912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H476"/>
+  <dimension ref="A1:H664"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="8" width="9.140625" style="1"/>
@@ -2690,7 +2750,7 @@
         <v>18</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -2701,13 +2761,13 @@
         <v>3</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -2718,13 +2778,13 @@
         <v>4</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -2735,13 +2795,13 @@
         <v>5</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -2752,13 +2812,13 @@
         <v>6</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -2775,7 +2835,7 @@
         <v>23</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -2786,7 +2846,7 @@
         <v>8</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D99" s="1" t="s">
         <v>24</v>
@@ -2797,12 +2857,12 @@
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="102" spans="1:8">
       <c r="B102" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C102" s="2" t="s">
         <v>34</v>
@@ -3059,12 +3119,12 @@
     </row>
     <row r="113" spans="1:8">
       <c r="A113" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="114" spans="1:8">
       <c r="B114" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C114" s="2" t="s">
         <v>34</v>
@@ -3321,12 +3381,12 @@
     </row>
     <row r="125" spans="1:8">
       <c r="A125" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="126" spans="1:8">
       <c r="B126" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C126" s="2" t="s">
         <v>34</v>
@@ -3583,7 +3643,7 @@
     </row>
     <row r="137" spans="1:8">
       <c r="A137" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="138" spans="1:8">
@@ -4151,7 +4211,7 @@
     </row>
     <row r="167" spans="1:7">
       <c r="A167" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -4176,7 +4236,7 @@
         <v>1</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D169" s="1" t="s">
         <v>17</v>
@@ -4193,13 +4253,13 @@
         <v>2</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D170" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="171" spans="1:7">
@@ -4210,13 +4270,13 @@
         <v>3</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="D171" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="172" spans="1:7">
@@ -4227,13 +4287,13 @@
         <v>4</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D172" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="173" spans="1:7">
@@ -4244,13 +4304,13 @@
         <v>5</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D173" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E173" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="174" spans="1:7">
@@ -4261,13 +4321,13 @@
         <v>6</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D174" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E174" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="175" spans="1:7">
@@ -4284,7 +4344,7 @@
         <v>23</v>
       </c>
       <c r="E175" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="176" spans="1:7">
@@ -4295,7 +4355,7 @@
         <v>8</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D176" s="1" t="s">
         <v>24</v>
@@ -4306,7 +4366,7 @@
     </row>
     <row r="178" spans="1:7">
       <c r="A178" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="179" spans="1:7">
@@ -4317,10 +4377,10 @@
         <v>35</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F179" s="2" t="s">
         <v>38</v>
@@ -4492,7 +4552,7 @@
     </row>
     <row r="188" spans="1:7">
       <c r="A188" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="189" spans="1:7">
@@ -4654,7 +4714,7 @@
     </row>
     <row r="198" spans="1:6">
       <c r="A198" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="199" spans="1:6">
@@ -4679,7 +4739,7 @@
         <v>1</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D200" s="1" t="s">
         <v>17</v>
@@ -4696,13 +4756,13 @@
         <v>2</v>
       </c>
       <c r="C201" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D201" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E201" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="202" spans="1:6">
@@ -4713,13 +4773,13 @@
         <v>3</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="D202" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E202" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="203" spans="1:6">
@@ -4730,13 +4790,13 @@
         <v>4</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D203" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E203" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="204" spans="1:6">
@@ -4747,13 +4807,13 @@
         <v>5</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D204" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E204" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="205" spans="1:6">
@@ -4764,13 +4824,13 @@
         <v>6</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D205" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E205" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="206" spans="1:6">
@@ -4787,7 +4847,7 @@
         <v>23</v>
       </c>
       <c r="E206" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="207" spans="1:6">
@@ -4798,7 +4858,7 @@
         <v>8</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D207" s="1" t="s">
         <v>24</v>
@@ -4809,7 +4869,7 @@
     </row>
     <row r="209" spans="1:7">
       <c r="A209" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="210" spans="1:7">
@@ -4820,10 +4880,10 @@
         <v>35</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E210" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F210" s="2" t="s">
         <v>38</v>
@@ -4880,7 +4940,7 @@
     </row>
     <row r="213" spans="1:7">
       <c r="A213" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B213" s="1">
         <v>-1.11558867186674</v>
@@ -4995,7 +5055,7 @@
     </row>
     <row r="219" spans="1:7">
       <c r="A219" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="220" spans="1:7">
@@ -5077,7 +5137,7 @@
     </row>
     <row r="224" spans="1:7">
       <c r="A224" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B224" s="1">
         <v>0.2824771975296116</v>
@@ -5154,7 +5214,7 @@
     </row>
     <row r="229" spans="1:6">
       <c r="A229" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="230" spans="1:6">
@@ -5179,7 +5239,7 @@
         <v>1</v>
       </c>
       <c r="C231" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D231" s="1" t="s">
         <v>17</v>
@@ -5196,13 +5256,13 @@
         <v>2</v>
       </c>
       <c r="C232" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D232" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E232" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="233" spans="1:6">
@@ -5213,13 +5273,13 @@
         <v>3</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="D233" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E233" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="234" spans="1:6">
@@ -5230,13 +5290,13 @@
         <v>4</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D234" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E234" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="235" spans="1:6">
@@ -5247,13 +5307,13 @@
         <v>5</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D235" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E235" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="236" spans="1:6">
@@ -5264,13 +5324,13 @@
         <v>6</v>
       </c>
       <c r="C236" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D236" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E236" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="237" spans="1:6">
@@ -5287,7 +5347,7 @@
         <v>23</v>
       </c>
       <c r="E237" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="238" spans="1:6">
@@ -5309,7 +5369,7 @@
     </row>
     <row r="240" spans="1:6">
       <c r="A240" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="241" spans="1:7">
@@ -5320,10 +5380,10 @@
         <v>35</v>
       </c>
       <c r="D241" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E241" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F241" s="2" t="s">
         <v>38</v>
@@ -5357,7 +5417,7 @@
     </row>
     <row r="243" spans="1:7">
       <c r="A243" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B243" s="1">
         <v>2.475108324951747</v>
@@ -5403,7 +5463,7 @@
     </row>
     <row r="245" spans="1:7">
       <c r="A245" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B245" s="1">
         <v>1.172146522488462</v>
@@ -5426,7 +5486,7 @@
     </row>
     <row r="247" spans="1:7">
       <c r="A247" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="248" spans="1:7">
@@ -5468,7 +5528,7 @@
     </row>
     <row r="250" spans="1:7">
       <c r="A250" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B250" s="1">
         <v>0.0004389868297785795</v>
@@ -5488,7 +5548,7 @@
     </row>
     <row r="251" spans="1:7">
       <c r="A251" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B251" s="1">
         <v>0.03919733536927187</v>
@@ -5528,7 +5588,7 @@
     </row>
     <row r="254" spans="1:7">
       <c r="A254" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="255" spans="1:7">
@@ -5570,7 +5630,7 @@
         <v>2</v>
       </c>
       <c r="C257" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D257" s="1" t="s">
         <v>18</v>
@@ -5587,7 +5647,7 @@
         <v>3</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="D258" s="1" t="s">
         <v>19</v>
@@ -5672,7 +5732,7 @@
         <v>8</v>
       </c>
       <c r="C263" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D263" s="1" t="s">
         <v>24</v>
@@ -6075,10 +6135,10 @@
     </row>
     <row r="281" spans="1:8">
       <c r="A281" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C281" s="1">
         <v>0.132899369457811</v>
@@ -6519,10 +6579,10 @@
     </row>
     <row r="300" spans="1:8">
       <c r="A300" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C300" s="1">
         <v>0.1221421410218785</v>
@@ -6963,10 +7023,10 @@
     </row>
     <row r="319" spans="1:8">
       <c r="A319" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C319" s="1">
         <v>0.2552177671192801</v>
@@ -7407,10 +7467,10 @@
     </row>
     <row r="338" spans="1:8">
       <c r="A338" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B338" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C338" s="1">
         <v>0.4220748693433146</v>
@@ -7851,10 +7911,10 @@
     </row>
     <row r="357" spans="1:8">
       <c r="A357" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C357" s="1">
         <v>0.1773128236392056</v>
@@ -8295,10 +8355,10 @@
     </row>
     <row r="376" spans="1:8">
       <c r="A376" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C376" s="1">
         <v>-0.2548184232345599</v>
@@ -8561,7 +8621,7 @@
     <row r="391" spans="1:7">
       <c r="A391" s="2"/>
       <c r="B391" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C391" s="1">
         <v>0.3243426031463325</v>
@@ -8878,7 +8938,7 @@
     <row r="407" spans="1:7">
       <c r="A407" s="2"/>
       <c r="B407" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C407" s="1">
         <v>0.4183881489014909</v>
@@ -9192,7 +9252,7 @@
     <row r="423" spans="1:7">
       <c r="A423" s="2"/>
       <c r="B423" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C423" s="1">
         <v>0.1147765647959176</v>
@@ -9500,7 +9560,7 @@
     <row r="439" spans="1:7">
       <c r="A439" s="2"/>
       <c r="B439" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C439" s="1">
         <v>0.009820048795527999</v>
@@ -9817,7 +9877,7 @@
     <row r="455" spans="1:7">
       <c r="A455" s="2"/>
       <c r="B455" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C455" s="1">
         <v>0.3090265089901769</v>
@@ -10125,7 +10185,7 @@
     <row r="471" spans="1:7">
       <c r="A471" s="2"/>
       <c r="B471" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C471" s="1">
         <v>0.552131630609431</v>
@@ -10236,8 +10296,3893 @@
         <v>2.136383465068589</v>
       </c>
     </row>
+    <row r="478" spans="1:7">
+      <c r="A478" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="479" spans="1:7">
+      <c r="B479" s="2">
+        <v>0</v>
+      </c>
+      <c r="C479" s="2">
+        <v>1</v>
+      </c>
+      <c r="D479" s="2">
+        <v>2</v>
+      </c>
+      <c r="E479" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="480" spans="1:7">
+      <c r="A480" s="2">
+        <v>0</v>
+      </c>
+      <c r="B480" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C480" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D480" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E480" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="481" spans="1:8">
+      <c r="A481" s="2">
+        <v>1</v>
+      </c>
+      <c r="B481" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C481" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D481" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E481" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="482" spans="1:8">
+      <c r="A482" s="2">
+        <v>2</v>
+      </c>
+      <c r="B482" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C482" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D482" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E482" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="483" spans="1:8">
+      <c r="A483" s="2">
+        <v>3</v>
+      </c>
+      <c r="B483" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C483" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D483" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E483" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="484" spans="1:8">
+      <c r="A484" s="2">
+        <v>4</v>
+      </c>
+      <c r="B484" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C484" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D484" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E484" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="485" spans="1:8">
+      <c r="A485" s="2">
+        <v>5</v>
+      </c>
+      <c r="B485" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C485" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D485" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E485" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="486" spans="1:8">
+      <c r="A486" s="2">
+        <v>6</v>
+      </c>
+      <c r="B486" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C486" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D486" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E486" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="487" spans="1:8">
+      <c r="A487" s="2">
+        <v>7</v>
+      </c>
+      <c r="B487" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C487" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D487" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E487" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="489" spans="1:8">
+      <c r="A489" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="490" spans="1:8">
+      <c r="B490" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C490" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D490" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E490" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F490" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G490" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H490" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="491" spans="1:8">
+      <c r="A491" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B491" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C491" s="1">
+        <v>0.2249915310175884</v>
+      </c>
+      <c r="D491" s="1">
+        <v>0.103953880740101</v>
+      </c>
+      <c r="E491" s="1">
+        <v>2.164339892034413</v>
+      </c>
+      <c r="F491" s="1">
+        <v>0.03043827325881311</v>
+      </c>
+      <c r="G491" s="1">
+        <v>0.02124566871381847</v>
+      </c>
+      <c r="H491" s="1">
+        <v>0.4287373933213583</v>
+      </c>
+    </row>
+    <row r="492" spans="1:8">
+      <c r="A492" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B492" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C492" s="1">
+        <v>0.1720144409370326</v>
+      </c>
+      <c r="D492" s="1">
+        <v>0.104765067980059</v>
+      </c>
+      <c r="E492" s="1">
+        <v>1.641906450819788</v>
+      </c>
+      <c r="F492" s="1">
+        <v>0.1006093927893698</v>
+      </c>
+      <c r="G492" s="1">
+        <v>-0.03332131914177355</v>
+      </c>
+      <c r="H492" s="1">
+        <v>0.3773502010158387</v>
+      </c>
+    </row>
+    <row r="493" spans="1:8">
+      <c r="A493" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B493" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C493" s="1">
+        <v>-0.07852664660079063</v>
+      </c>
+      <c r="D493" s="1">
+        <v>0.09589490935179851</v>
+      </c>
+      <c r="E493" s="1">
+        <v>-0.8188823278690327</v>
+      </c>
+      <c r="F493" s="1">
+        <v>0.4128535534896671</v>
+      </c>
+      <c r="G493" s="1">
+        <v>-0.2664772152310489</v>
+      </c>
+      <c r="H493" s="1">
+        <v>0.1094239220294677</v>
+      </c>
+    </row>
+    <row r="494" spans="1:8">
+      <c r="A494" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B494" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C494" s="1">
+        <v>0.213347653103811</v>
+      </c>
+      <c r="D494" s="1">
+        <v>0.1383477753656325</v>
+      </c>
+      <c r="E494" s="1">
+        <v>1.542111194343133</v>
+      </c>
+      <c r="F494" s="1">
+        <v>0.1230465751327812</v>
+      </c>
+      <c r="G494" s="1">
+        <v>-0.05780900395406638</v>
+      </c>
+      <c r="H494" s="1">
+        <v>0.4845043101616884</v>
+      </c>
+    </row>
+    <row r="495" spans="1:8">
+      <c r="A495" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B495" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C495" s="1">
+        <v>-0.0975134458701325</v>
+      </c>
+      <c r="D495" s="1">
+        <v>0.235669782311117</v>
+      </c>
+      <c r="E495" s="1">
+        <v>-0.4137715277447032</v>
+      </c>
+      <c r="F495" s="1">
+        <v>0.679041437636994</v>
+      </c>
+      <c r="G495" s="1">
+        <v>-0.5594177314443165</v>
+      </c>
+      <c r="H495" s="1">
+        <v>0.3643908397040515</v>
+      </c>
+    </row>
+    <row r="496" spans="1:8">
+      <c r="A496" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B496" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C496" s="1">
+        <v>-0.525759190566162</v>
+      </c>
+      <c r="D496" s="1">
+        <v>0.1475290550568114</v>
+      </c>
+      <c r="E496" s="1">
+        <v>-3.56376708549851</v>
+      </c>
+      <c r="F496" s="1">
+        <v>0.0003655703611464461</v>
+      </c>
+      <c r="G496" s="1">
+        <v>-0.8149108251507392</v>
+      </c>
+      <c r="H496" s="1">
+        <v>-0.2366075559815849</v>
+      </c>
+    </row>
+    <row r="497" spans="1:8">
+      <c r="A497" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B497" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C497" s="1">
+        <v>-0.1008073201356094</v>
+      </c>
+      <c r="D497" s="1">
+        <v>0.09546461901523623</v>
+      </c>
+      <c r="E497" s="1">
+        <v>-1.055965248439534</v>
+      </c>
+      <c r="F497" s="1">
+        <v>0.2909840920523293</v>
+      </c>
+      <c r="G497" s="1">
+        <v>-0.28791453520331</v>
+      </c>
+      <c r="H497" s="1">
+        <v>0.08629989493209123</v>
+      </c>
+    </row>
+    <row r="498" spans="1:8">
+      <c r="A498" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B498" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C498" s="1">
+        <v>-0.2458702992489558</v>
+      </c>
+      <c r="D498" s="1">
+        <v>0.09664387816431816</v>
+      </c>
+      <c r="E498" s="1">
+        <v>-2.544085604997312</v>
+      </c>
+      <c r="F498" s="1">
+        <v>0.01095642293665167</v>
+      </c>
+      <c r="G498" s="1">
+        <v>-0.4352888197772964</v>
+      </c>
+      <c r="H498" s="1">
+        <v>-0.0564517787206153</v>
+      </c>
+    </row>
+    <row r="499" spans="1:8">
+      <c r="A499" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B499" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C499" s="1">
+        <v>-0.8785684007948122</v>
+      </c>
+      <c r="D499" s="1">
+        <v>0.09649497345459762</v>
+      </c>
+      <c r="E499" s="1">
+        <v>-9.104810015914376</v>
+      </c>
+      <c r="F499" s="1">
+        <v>8.641755080100111E-20</v>
+      </c>
+      <c r="G499" s="1">
+        <v>-1.067695073454972</v>
+      </c>
+      <c r="H499" s="1">
+        <v>-0.6894417281346523</v>
+      </c>
+    </row>
+    <row r="500" spans="1:8">
+      <c r="A500" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B500" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C500" s="1">
+        <v>-0.08132550156481841</v>
+      </c>
+      <c r="D500" s="1">
+        <v>0.1382832423833657</v>
+      </c>
+      <c r="E500" s="1">
+        <v>-0.5881081479081747</v>
+      </c>
+      <c r="F500" s="1">
+        <v>0.5564597044586419</v>
+      </c>
+      <c r="G500" s="1">
+        <v>-0.3523556763016379</v>
+      </c>
+      <c r="H500" s="1">
+        <v>0.1897046731720011</v>
+      </c>
+    </row>
+    <row r="501" spans="1:8">
+      <c r="A501" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B501" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C501" s="1">
+        <v>-1.345701620395633</v>
+      </c>
+      <c r="D501" s="1">
+        <v>0.5382528342111568</v>
+      </c>
+      <c r="E501" s="1">
+        <v>-2.500129186254715</v>
+      </c>
+      <c r="F501" s="1">
+        <v>0.01241480255182997</v>
+      </c>
+      <c r="G501" s="1">
+        <v>-2.400657790026109</v>
+      </c>
+      <c r="H501" s="1">
+        <v>-0.2907454507651572</v>
+      </c>
+    </row>
+    <row r="502" spans="1:8">
+      <c r="A502" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B502" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C502" s="1">
+        <v>-0.09975885052689878</v>
+      </c>
+      <c r="D502" s="1">
+        <v>0.1318545116874724</v>
+      </c>
+      <c r="E502" s="1">
+        <v>-0.7565827611826567</v>
+      </c>
+      <c r="F502" s="1">
+        <v>0.4492998724301147</v>
+      </c>
+      <c r="G502" s="1">
+        <v>-0.3581889446334604</v>
+      </c>
+      <c r="H502" s="1">
+        <v>0.1586712435796629</v>
+      </c>
+    </row>
+    <row r="503" spans="1:8">
+      <c r="A503" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B503" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C503" s="1">
+        <v>-0.5144379452912305</v>
+      </c>
+      <c r="D503" s="1">
+        <v>0.1815404455641338</v>
+      </c>
+      <c r="E503" s="1">
+        <v>-2.833737372917773</v>
+      </c>
+      <c r="F503" s="1">
+        <v>0.004600712496250168</v>
+      </c>
+      <c r="G503" s="1">
+        <v>-0.870250680334287</v>
+      </c>
+      <c r="H503" s="1">
+        <v>-0.1586252102481741</v>
+      </c>
+    </row>
+    <row r="505" spans="1:8">
+      <c r="A505" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="506" spans="1:8">
+      <c r="B506" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C506" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D506" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E506" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F506" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G506" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H506" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="507" spans="1:8">
+      <c r="A507" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B507" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C507" s="1">
+        <v>-1.564522656474258</v>
+      </c>
+      <c r="D507" s="1">
+        <v>0.1268952915924901</v>
+      </c>
+      <c r="E507" s="1">
+        <v>-12.32924119437422</v>
+      </c>
+      <c r="F507" s="1">
+        <v>6.303753463585649E-35</v>
+      </c>
+      <c r="G507" s="1">
+        <v>-1.813232857803247</v>
+      </c>
+      <c r="H507" s="1">
+        <v>-1.315812455145269</v>
+      </c>
+    </row>
+    <row r="508" spans="1:8">
+      <c r="A508" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B508" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C508" s="1">
+        <v>-0.2751810024799334</v>
+      </c>
+      <c r="D508" s="1">
+        <v>0.1098995809319774</v>
+      </c>
+      <c r="E508" s="1">
+        <v>-2.503931317538484</v>
+      </c>
+      <c r="F508" s="1">
+        <v>0.01228218742131392</v>
+      </c>
+      <c r="G508" s="1">
+        <v>-0.490580223022654</v>
+      </c>
+      <c r="H508" s="1">
+        <v>-0.05978178193721284</v>
+      </c>
+    </row>
+    <row r="509" spans="1:8">
+      <c r="A509" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B509" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C509" s="1">
+        <v>0.3520332992925154</v>
+      </c>
+      <c r="D509" s="1">
+        <v>0.09125598429002252</v>
+      </c>
+      <c r="E509" s="1">
+        <v>3.857646181029741</v>
+      </c>
+      <c r="F509" s="1">
+        <v>0.0001144842107323911</v>
+      </c>
+      <c r="G509" s="1">
+        <v>0.1731748567103183</v>
+      </c>
+      <c r="H509" s="1">
+        <v>0.5308917418747126</v>
+      </c>
+    </row>
+    <row r="510" spans="1:8">
+      <c r="A510" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B510" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C510" s="1">
+        <v>-0.6150788002864479</v>
+      </c>
+      <c r="D510" s="1">
+        <v>0.20272506463271</v>
+      </c>
+      <c r="E510" s="1">
+        <v>-3.034054034713594</v>
+      </c>
+      <c r="F510" s="1">
+        <v>0.002412912081644074</v>
+      </c>
+      <c r="G510" s="1">
+        <v>-1.012412625730114</v>
+      </c>
+      <c r="H510" s="1">
+        <v>-0.2177449748427815</v>
+      </c>
+    </row>
+    <row r="511" spans="1:8">
+      <c r="A511" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B511" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C511" s="1">
+        <v>-0.3205837031620951</v>
+      </c>
+      <c r="D511" s="1">
+        <v>0.2666424776891327</v>
+      </c>
+      <c r="E511" s="1">
+        <v>-1.202297945700348</v>
+      </c>
+      <c r="F511" s="1">
+        <v>0.2292481125687863</v>
+      </c>
+      <c r="G511" s="1">
+        <v>-0.8431933561813201</v>
+      </c>
+      <c r="H511" s="1">
+        <v>0.2020259498571299</v>
+      </c>
+    </row>
+    <row r="512" spans="1:8">
+      <c r="A512" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B512" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C512" s="1">
+        <v>0.599932705289018</v>
+      </c>
+      <c r="D512" s="1">
+        <v>0.1063692071787075</v>
+      </c>
+      <c r="E512" s="1">
+        <v>5.640097554559095</v>
+      </c>
+      <c r="F512" s="1">
+        <v>1.699538476781488E-08</v>
+      </c>
+      <c r="G512" s="1">
+        <v>0.3914528901546719</v>
+      </c>
+      <c r="H512" s="1">
+        <v>0.8084125204233641</v>
+      </c>
+    </row>
+    <row r="513" spans="1:8">
+      <c r="A513" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B513" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C513" s="1">
+        <v>0.174499156682957</v>
+      </c>
+      <c r="D513" s="1">
+        <v>0.08870653098542031</v>
+      </c>
+      <c r="E513" s="1">
+        <v>1.967151175279726</v>
+      </c>
+      <c r="F513" s="1">
+        <v>0.0491657849146158</v>
+      </c>
+      <c r="G513" s="1">
+        <v>0.000637550758046862</v>
+      </c>
+      <c r="H513" s="1">
+        <v>0.3483607626078672</v>
+      </c>
+    </row>
+    <row r="514" spans="1:8">
+      <c r="A514" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B514" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C514" s="1">
+        <v>0.07792513011951603</v>
+      </c>
+      <c r="D514" s="1">
+        <v>0.1038844712090115</v>
+      </c>
+      <c r="E514" s="1">
+        <v>0.7501133635529967</v>
+      </c>
+      <c r="F514" s="1">
+        <v>0.4531864316378061</v>
+      </c>
+      <c r="G514" s="1">
+        <v>-0.1256846920031346</v>
+      </c>
+      <c r="H514" s="1">
+        <v>0.2815349522421666</v>
+      </c>
+    </row>
+    <row r="515" spans="1:8">
+      <c r="A515" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B515" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C515" s="1">
+        <v>1.262442661138902</v>
+      </c>
+      <c r="D515" s="1">
+        <v>0.104279670996257</v>
+      </c>
+      <c r="E515" s="1">
+        <v>12.1063161120274</v>
+      </c>
+      <c r="F515" s="1">
+        <v>9.778824029820875E-34</v>
+      </c>
+      <c r="G515" s="1">
+        <v>1.058058261666552</v>
+      </c>
+      <c r="H515" s="1">
+        <v>1.466827060611252</v>
+      </c>
+    </row>
+    <row r="516" spans="1:8">
+      <c r="A516" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B516" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C516" s="1">
+        <v>0.7258116961408411</v>
+      </c>
+      <c r="D516" s="1">
+        <v>0.1044928608339838</v>
+      </c>
+      <c r="E516" s="1">
+        <v>6.946041005557272</v>
+      </c>
+      <c r="F516" s="1">
+        <v>3.756796141150703E-12</v>
+      </c>
+      <c r="G516" s="1">
+        <v>0.5210094522646768</v>
+      </c>
+      <c r="H516" s="1">
+        <v>0.9306139400170054</v>
+      </c>
+    </row>
+    <row r="517" spans="1:8">
+      <c r="A517" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B517" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C517" s="1">
+        <v>0.3476180579097375</v>
+      </c>
+      <c r="D517" s="1">
+        <v>0.2336072475304196</v>
+      </c>
+      <c r="E517" s="1">
+        <v>1.488044834158974</v>
+      </c>
+      <c r="F517" s="1">
+        <v>0.1367390703151118</v>
+      </c>
+      <c r="G517" s="1">
+        <v>-0.1102437337774183</v>
+      </c>
+      <c r="H517" s="1">
+        <v>0.8054798495968933</v>
+      </c>
+    </row>
+    <row r="518" spans="1:8">
+      <c r="A518" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B518" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C518" s="1">
+        <v>-0.01724535193601182</v>
+      </c>
+      <c r="D518" s="1">
+        <v>0.1242742669182388</v>
+      </c>
+      <c r="E518" s="1">
+        <v>-0.1387684865391939</v>
+      </c>
+      <c r="F518" s="1">
+        <v>0.8896330971005005</v>
+      </c>
+      <c r="G518" s="1">
+        <v>-0.2608184393008774</v>
+      </c>
+      <c r="H518" s="1">
+        <v>0.2263277354288538</v>
+      </c>
+    </row>
+    <row r="519" spans="1:8">
+      <c r="A519" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B519" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C519" s="1">
+        <v>-0.02898443468592734</v>
+      </c>
+      <c r="D519" s="1">
+        <v>0.1354511552089917</v>
+      </c>
+      <c r="E519" s="1">
+        <v>-0.2139844037594687</v>
+      </c>
+      <c r="F519" s="1">
+        <v>0.83055921949477</v>
+      </c>
+      <c r="G519" s="1">
+        <v>-0.294463820559896</v>
+      </c>
+      <c r="H519" s="1">
+        <v>0.2364949511880413</v>
+      </c>
+    </row>
+    <row r="521" spans="1:8">
+      <c r="A521" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="522" spans="1:8">
+      <c r="B522" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C522" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D522" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E522" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F522" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G522" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H522" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="523" spans="1:8">
+      <c r="A523" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B523" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C523" s="1">
+        <v>-1.285838296902032</v>
+      </c>
+      <c r="D523" s="1">
+        <v>0.1311472820027768</v>
+      </c>
+      <c r="E523" s="1">
+        <v>-9.804536375178605</v>
+      </c>
+      <c r="F523" s="1">
+        <v>1.076401634377507E-22</v>
+      </c>
+      <c r="G523" s="1">
+        <v>-1.542882246297792</v>
+      </c>
+      <c r="H523" s="1">
+        <v>-1.028794347506271</v>
+      </c>
+    </row>
+    <row r="524" spans="1:8">
+      <c r="A524" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B524" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C524" s="1">
+        <v>-0.2121496299955544</v>
+      </c>
+      <c r="D524" s="1">
+        <v>0.1269000986881279</v>
+      </c>
+      <c r="E524" s="1">
+        <v>-1.671784594249508</v>
+      </c>
+      <c r="F524" s="1">
+        <v>0.09456680576091746</v>
+      </c>
+      <c r="G524" s="1">
+        <v>-0.4608692530588636</v>
+      </c>
+      <c r="H524" s="1">
+        <v>0.03656999306775477</v>
+      </c>
+    </row>
+    <row r="525" spans="1:8">
+      <c r="A525" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B525" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C525" s="1">
+        <v>0.1785060895041023</v>
+      </c>
+      <c r="D525" s="1">
+        <v>0.1054426663177848</v>
+      </c>
+      <c r="E525" s="1">
+        <v>1.692920861524098</v>
+      </c>
+      <c r="F525" s="1">
+        <v>0.09047053184849052</v>
+      </c>
+      <c r="G525" s="1">
+        <v>-0.02815773891263063</v>
+      </c>
+      <c r="H525" s="1">
+        <v>0.3851699179208352</v>
+      </c>
+    </row>
+    <row r="526" spans="1:8">
+      <c r="A526" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B526" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C526" s="1">
+        <v>-0.7164695252610598</v>
+      </c>
+      <c r="D526" s="1">
+        <v>0.2339286018208551</v>
+      </c>
+      <c r="E526" s="1">
+        <v>-3.062770091746795</v>
+      </c>
+      <c r="F526" s="1">
+        <v>0.002192984741371619</v>
+      </c>
+      <c r="G526" s="1">
+        <v>-1.174961159783747</v>
+      </c>
+      <c r="H526" s="1">
+        <v>-0.2579778907383729</v>
+      </c>
+    </row>
+    <row r="527" spans="1:8">
+      <c r="A527" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B527" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C527" s="1">
+        <v>0.1885684036585996</v>
+      </c>
+      <c r="D527" s="1">
+        <v>0.2587859989751609</v>
+      </c>
+      <c r="E527" s="1">
+        <v>0.7286654007765658</v>
+      </c>
+      <c r="F527" s="1">
+        <v>0.4662063620866697</v>
+      </c>
+      <c r="G527" s="1">
+        <v>-0.3186428340359351</v>
+      </c>
+      <c r="H527" s="1">
+        <v>0.6957796413531343</v>
+      </c>
+    </row>
+    <row r="528" spans="1:8">
+      <c r="A528" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B528" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C528" s="1">
+        <v>0.6004042002639752</v>
+      </c>
+      <c r="D528" s="1">
+        <v>0.1209533802064972</v>
+      </c>
+      <c r="E528" s="1">
+        <v>4.963930724705151</v>
+      </c>
+      <c r="F528" s="1">
+        <v>6.908059231390752E-07</v>
+      </c>
+      <c r="G528" s="1">
+        <v>0.3633399312508609</v>
+      </c>
+      <c r="H528" s="1">
+        <v>0.8374684692770895</v>
+      </c>
+    </row>
+    <row r="529" spans="1:8">
+      <c r="A529" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B529" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C529" s="1">
+        <v>-0.1580344194412602</v>
+      </c>
+      <c r="D529" s="1">
+        <v>0.1047321434260525</v>
+      </c>
+      <c r="E529" s="1">
+        <v>-1.508939035061786</v>
+      </c>
+      <c r="F529" s="1">
+        <v>0.131314363173481</v>
+      </c>
+      <c r="G529" s="1">
+        <v>-0.3633056485800066</v>
+      </c>
+      <c r="H529" s="1">
+        <v>0.04723680969748609</v>
+      </c>
+    </row>
+    <row r="530" spans="1:8">
+      <c r="A530" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B530" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C530" s="1">
+        <v>-0.1430212518678175</v>
+      </c>
+      <c r="D530" s="1">
+        <v>0.1141747530555115</v>
+      </c>
+      <c r="E530" s="1">
+        <v>-1.252652167316542</v>
+      </c>
+      <c r="F530" s="1">
+        <v>0.2103323207642823</v>
+      </c>
+      <c r="G530" s="1">
+        <v>-0.3667996558003745</v>
+      </c>
+      <c r="H530" s="1">
+        <v>0.08075715206473952</v>
+      </c>
+    </row>
+    <row r="531" spans="1:8">
+      <c r="A531" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B531" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C531" s="1">
+        <v>0.533234381099385</v>
+      </c>
+      <c r="D531" s="1">
+        <v>0.1103218186410626</v>
+      </c>
+      <c r="E531" s="1">
+        <v>4.833444441613939</v>
+      </c>
+      <c r="F531" s="1">
+        <v>1.341907416072246E-06</v>
+      </c>
+      <c r="G531" s="1">
+        <v>0.3170075898539428</v>
+      </c>
+      <c r="H531" s="1">
+        <v>0.7494611723448272</v>
+      </c>
+    </row>
+    <row r="532" spans="1:8">
+      <c r="A532" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B532" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C532" s="1">
+        <v>1.023314050932608</v>
+      </c>
+      <c r="D532" s="1">
+        <v>0.1164189779738178</v>
+      </c>
+      <c r="E532" s="1">
+        <v>8.789924707660191</v>
+      </c>
+      <c r="F532" s="1">
+        <v>1.496602319378977E-18</v>
+      </c>
+      <c r="G532" s="1">
+        <v>0.7951370469869637</v>
+      </c>
+      <c r="H532" s="1">
+        <v>1.251491054878253</v>
+      </c>
+    </row>
+    <row r="533" spans="1:8">
+      <c r="A533" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B533" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C533" s="1">
+        <v>-0.1383993577784189</v>
+      </c>
+      <c r="D533" s="1">
+        <v>0.303679025727264</v>
+      </c>
+      <c r="E533" s="1">
+        <v>-0.4557422345747257</v>
+      </c>
+      <c r="F533" s="1">
+        <v>0.6485753473899263</v>
+      </c>
+      <c r="G533" s="1">
+        <v>-0.7335993110640689</v>
+      </c>
+      <c r="H533" s="1">
+        <v>0.4568005955072311</v>
+      </c>
+    </row>
+    <row r="534" spans="1:8">
+      <c r="A534" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B534" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C534" s="1">
+        <v>0.291266449624504</v>
+      </c>
+      <c r="D534" s="1">
+        <v>0.1405039440260273</v>
+      </c>
+      <c r="E534" s="1">
+        <v>2.073012623549905</v>
+      </c>
+      <c r="F534" s="1">
+        <v>0.03817110476886406</v>
+      </c>
+      <c r="G534" s="1">
+        <v>0.01588377964765875</v>
+      </c>
+      <c r="H534" s="1">
+        <v>0.5666491196013492</v>
+      </c>
+    </row>
+    <row r="535" spans="1:8">
+      <c r="A535" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B535" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C535" s="1">
+        <v>-0.3479353151065283</v>
+      </c>
+      <c r="D535" s="1">
+        <v>0.1739309024485958</v>
+      </c>
+      <c r="E535" s="1">
+        <v>-2.000422640303142</v>
+      </c>
+      <c r="F535" s="1">
+        <v>0.04545464566362853</v>
+      </c>
+      <c r="G535" s="1">
+        <v>-0.6888336197043256</v>
+      </c>
+      <c r="H535" s="1">
+        <v>-0.007037010508730956</v>
+      </c>
+    </row>
+    <row r="537" spans="1:8">
+      <c r="A537" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="538" spans="1:8">
+      <c r="B538" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C538" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D538" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E538" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F538" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G538" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H538" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="539" spans="1:8">
+      <c r="A539" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B539" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C539" s="1">
+        <v>-1.608813445389444</v>
+      </c>
+      <c r="D539" s="1">
+        <v>0.1414699763169429</v>
+      </c>
+      <c r="E539" s="1">
+        <v>-11.37211928123273</v>
+      </c>
+      <c r="F539" s="1">
+        <v>5.75724982403861E-30</v>
+      </c>
+      <c r="G539" s="1">
+        <v>-1.886089503864387</v>
+      </c>
+      <c r="H539" s="1">
+        <v>-1.331537386914502</v>
+      </c>
+    </row>
+    <row r="540" spans="1:8">
+      <c r="A540" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B540" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C540" s="1">
+        <v>0.154227424551831</v>
+      </c>
+      <c r="D540" s="1">
+        <v>0.1198855560981439</v>
+      </c>
+      <c r="E540" s="1">
+        <v>1.286455429422818</v>
+      </c>
+      <c r="F540" s="1">
+        <v>0.19828416430527</v>
+      </c>
+      <c r="G540" s="1">
+        <v>-0.08074394766708728</v>
+      </c>
+      <c r="H540" s="1">
+        <v>0.3891987967707493</v>
+      </c>
+    </row>
+    <row r="541" spans="1:8">
+      <c r="A541" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B541" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C541" s="1">
+        <v>0.09753952427747316</v>
+      </c>
+      <c r="D541" s="1">
+        <v>0.1077465967920705</v>
+      </c>
+      <c r="E541" s="1">
+        <v>0.905267796677653</v>
+      </c>
+      <c r="F541" s="1">
+        <v>0.3653235325354613</v>
+      </c>
+      <c r="G541" s="1">
+        <v>-0.113639924891744</v>
+      </c>
+      <c r="H541" s="1">
+        <v>0.3087189734466903</v>
+      </c>
+    </row>
+    <row r="542" spans="1:8">
+      <c r="A542" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B542" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C542" s="1">
+        <v>0.1000252205395829</v>
+      </c>
+      <c r="D542" s="1">
+        <v>0.1852392373633804</v>
+      </c>
+      <c r="E542" s="1">
+        <v>0.5399785810139418</v>
+      </c>
+      <c r="F542" s="1">
+        <v>0.5892118038207506</v>
+      </c>
+      <c r="G542" s="1">
+        <v>-0.263037013216309</v>
+      </c>
+      <c r="H542" s="1">
+        <v>0.4630874542954748</v>
+      </c>
+    </row>
+    <row r="543" spans="1:8">
+      <c r="A543" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B543" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C543" s="1">
+        <v>0.2876073902288768</v>
+      </c>
+      <c r="D543" s="1">
+        <v>0.2593859825735187</v>
+      </c>
+      <c r="E543" s="1">
+        <v>1.108800820211475</v>
+      </c>
+      <c r="F543" s="1">
+        <v>0.2675161165776037</v>
+      </c>
+      <c r="G543" s="1">
+        <v>-0.220779793709754</v>
+      </c>
+      <c r="H543" s="1">
+        <v>0.7959945741675076</v>
+      </c>
+    </row>
+    <row r="544" spans="1:8">
+      <c r="A544" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B544" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C544" s="1">
+        <v>0.1573664407356352</v>
+      </c>
+      <c r="D544" s="1">
+        <v>0.1355040510575941</v>
+      </c>
+      <c r="E544" s="1">
+        <v>1.161341225649031</v>
+      </c>
+      <c r="F544" s="1">
+        <v>0.2455031605052839</v>
+      </c>
+      <c r="G544" s="1">
+        <v>-0.1082166190965258</v>
+      </c>
+      <c r="H544" s="1">
+        <v>0.4229495005677962</v>
+      </c>
+    </row>
+    <row r="545" spans="1:8">
+      <c r="A545" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B545" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C545" s="1">
+        <v>0.006702317118651681</v>
+      </c>
+      <c r="D545" s="1">
+        <v>0.1047058391616192</v>
+      </c>
+      <c r="E545" s="1">
+        <v>0.06401092023441296</v>
+      </c>
+      <c r="F545" s="1">
+        <v>0.9489615315521314</v>
+      </c>
+      <c r="G545" s="1">
+        <v>-0.1985173566091656</v>
+      </c>
+      <c r="H545" s="1">
+        <v>0.2119219908464689</v>
+      </c>
+    </row>
+    <row r="546" spans="1:8">
+      <c r="A546" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B546" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C546" s="1">
+        <v>0.08888038077609614</v>
+      </c>
+      <c r="D546" s="1">
+        <v>0.1208520775446927</v>
+      </c>
+      <c r="E546" s="1">
+        <v>0.7354476859798048</v>
+      </c>
+      <c r="F546" s="1">
+        <v>0.4620668891808699</v>
+      </c>
+      <c r="G546" s="1">
+        <v>-0.1479853386683433</v>
+      </c>
+      <c r="H546" s="1">
+        <v>0.3257461002205355</v>
+      </c>
+    </row>
+    <row r="547" spans="1:8">
+      <c r="A547" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B547" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C547" s="1">
+        <v>0.7761601501414654</v>
+      </c>
+      <c r="D547" s="1">
+        <v>0.1136431490427941</v>
+      </c>
+      <c r="E547" s="1">
+        <v>6.829801503029366</v>
+      </c>
+      <c r="F547" s="1">
+        <v>8.503220591470087E-12</v>
+      </c>
+      <c r="G547" s="1">
+        <v>0.5534236709278715</v>
+      </c>
+      <c r="H547" s="1">
+        <v>0.9988966293550594</v>
+      </c>
+    </row>
+    <row r="548" spans="1:8">
+      <c r="A548" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B548" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C548" s="1">
+        <v>0.1495229487029993</v>
+      </c>
+      <c r="D548" s="1">
+        <v>0.1330276603822068</v>
+      </c>
+      <c r="E548" s="1">
+        <v>1.123998935810788</v>
+      </c>
+      <c r="F548" s="1">
+        <v>0.2610134774064551</v>
+      </c>
+      <c r="G548" s="1">
+        <v>-0.1112064745937517</v>
+      </c>
+      <c r="H548" s="1">
+        <v>0.4102523719997503</v>
+      </c>
+    </row>
+    <row r="549" spans="1:8">
+      <c r="A549" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B549" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C549" s="1">
+        <v>0.1355284035128653</v>
+      </c>
+      <c r="D549" s="1">
+        <v>0.2623993830032211</v>
+      </c>
+      <c r="E549" s="1">
+        <v>0.5164966546861186</v>
+      </c>
+      <c r="F549" s="1">
+        <v>0.6055075748093981</v>
+      </c>
+      <c r="G549" s="1">
+        <v>-0.3787649367389797</v>
+      </c>
+      <c r="H549" s="1">
+        <v>0.6498217437647102</v>
+      </c>
+    </row>
+    <row r="550" spans="1:8">
+      <c r="A550" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B550" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C550" s="1">
+        <v>0.129542118501986</v>
+      </c>
+      <c r="D550" s="1">
+        <v>0.1385908124910919</v>
+      </c>
+      <c r="E550" s="1">
+        <v>0.9347092795946523</v>
+      </c>
+      <c r="F550" s="1">
+        <v>0.3499381433206767</v>
+      </c>
+      <c r="G550" s="1">
+        <v>-0.1420908825686979</v>
+      </c>
+      <c r="H550" s="1">
+        <v>0.40117511957267</v>
+      </c>
+    </row>
+    <row r="551" spans="1:8">
+      <c r="A551" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B551" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C551" s="1">
+        <v>0.1313752178525543</v>
+      </c>
+      <c r="D551" s="1">
+        <v>0.1520212273213681</v>
+      </c>
+      <c r="E551" s="1">
+        <v>0.8641899566751379</v>
+      </c>
+      <c r="F551" s="1">
+        <v>0.3874835484867725</v>
+      </c>
+      <c r="G551" s="1">
+        <v>-0.1665809125829035</v>
+      </c>
+      <c r="H551" s="1">
+        <v>0.4293313482880122</v>
+      </c>
+    </row>
+    <row r="553" spans="1:8">
+      <c r="A553" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="554" spans="1:8">
+      <c r="B554" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C554" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D554" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E554" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F554" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G554" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H554" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="555" spans="1:8">
+      <c r="A555" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B555" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C555" s="1">
+        <v>-1.347728288940703</v>
+      </c>
+      <c r="D555" s="1">
+        <v>0.1387446624185872</v>
+      </c>
+      <c r="E555" s="1">
+        <v>-9.713730715453828</v>
+      </c>
+      <c r="F555" s="1">
+        <v>2.635115730555844E-22</v>
+      </c>
+      <c r="G555" s="1">
+        <v>-1.619662830328301</v>
+      </c>
+      <c r="H555" s="1">
+        <v>-1.075793747553104</v>
+      </c>
+    </row>
+    <row r="556" spans="1:8">
+      <c r="A556" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B556" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C556" s="1">
+        <v>-0.04163407751758721</v>
+      </c>
+      <c r="D556" s="1">
+        <v>0.1322882452205772</v>
+      </c>
+      <c r="E556" s="1">
+        <v>-0.3147224263816232</v>
+      </c>
+      <c r="F556" s="1">
+        <v>0.7529724151289838</v>
+      </c>
+      <c r="G556" s="1">
+        <v>-0.3009142737279213</v>
+      </c>
+      <c r="H556" s="1">
+        <v>0.2176461186927469</v>
+      </c>
+    </row>
+    <row r="557" spans="1:8">
+      <c r="A557" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B557" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C557" s="1">
+        <v>0.304569205652149</v>
+      </c>
+      <c r="D557" s="1">
+        <v>0.1133375920597473</v>
+      </c>
+      <c r="E557" s="1">
+        <v>2.687274364286756</v>
+      </c>
+      <c r="F557" s="1">
+        <v>0.007203775417692744</v>
+      </c>
+      <c r="G557" s="1">
+        <v>0.08243160712055156</v>
+      </c>
+      <c r="H557" s="1">
+        <v>0.5267068041837465</v>
+      </c>
+    </row>
+    <row r="558" spans="1:8">
+      <c r="A558" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B558" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C558" s="1">
+        <v>-0.4877078073534579</v>
+      </c>
+      <c r="D558" s="1">
+        <v>0.2234224874805275</v>
+      </c>
+      <c r="E558" s="1">
+        <v>-2.182894895017961</v>
+      </c>
+      <c r="F558" s="1">
+        <v>0.02904355107345591</v>
+      </c>
+      <c r="G558" s="1">
+        <v>-0.9256078361516429</v>
+      </c>
+      <c r="H558" s="1">
+        <v>-0.0498077785552728</v>
+      </c>
+    </row>
+    <row r="559" spans="1:8">
+      <c r="A559" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B559" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C559" s="1">
+        <v>-0.175897156978274</v>
+      </c>
+      <c r="D559" s="1">
+        <v>0.311396529884221</v>
+      </c>
+      <c r="E559" s="1">
+        <v>-0.5648655013711088</v>
+      </c>
+      <c r="F559" s="1">
+        <v>0.5721652503803307</v>
+      </c>
+      <c r="G559" s="1">
+        <v>-0.7862231404620978</v>
+      </c>
+      <c r="H559" s="1">
+        <v>0.4344288265055499</v>
+      </c>
+    </row>
+    <row r="560" spans="1:8">
+      <c r="A560" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B560" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C560" s="1">
+        <v>0.6569371090209135</v>
+      </c>
+      <c r="D560" s="1">
+        <v>0.1310466025230827</v>
+      </c>
+      <c r="E560" s="1">
+        <v>5.01300374349804</v>
+      </c>
+      <c r="F560" s="1">
+        <v>5.358685390828512E-07</v>
+      </c>
+      <c r="G560" s="1">
+        <v>0.4000904877793356</v>
+      </c>
+      <c r="H560" s="1">
+        <v>0.9137837302624914</v>
+      </c>
+    </row>
+    <row r="561" spans="1:8">
+      <c r="A561" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B561" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C561" s="1">
+        <v>0.05300476067247347</v>
+      </c>
+      <c r="D561" s="1">
+        <v>0.1128499364410048</v>
+      </c>
+      <c r="E561" s="1">
+        <v>0.4696924282290854</v>
+      </c>
+      <c r="F561" s="1">
+        <v>0.6385747782972211</v>
+      </c>
+      <c r="G561" s="1">
+        <v>-0.16817705040953</v>
+      </c>
+      <c r="H561" s="1">
+        <v>0.274186571754477</v>
+      </c>
+    </row>
+    <row r="562" spans="1:8">
+      <c r="A562" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B562" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C562" s="1">
+        <v>-0.04264627882691358</v>
+      </c>
+      <c r="D562" s="1">
+        <v>0.1239023550325133</v>
+      </c>
+      <c r="E562" s="1">
+        <v>-0.3441926411787957</v>
+      </c>
+      <c r="F562" s="1">
+        <v>0.7307014160917791</v>
+      </c>
+      <c r="G562" s="1">
+        <v>-0.2854904322903347</v>
+      </c>
+      <c r="H562" s="1">
+        <v>0.2001978746365075</v>
+      </c>
+    </row>
+    <row r="563" spans="1:8">
+      <c r="A563" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B563" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C563" s="1">
+        <v>0.1128019117950421</v>
+      </c>
+      <c r="D563" s="1">
+        <v>0.1143875374259375</v>
+      </c>
+      <c r="E563" s="1">
+        <v>0.9861381260006405</v>
+      </c>
+      <c r="F563" s="1">
+        <v>0.3240653368093933</v>
+      </c>
+      <c r="G563" s="1">
+        <v>-0.1113935418400228</v>
+      </c>
+      <c r="H563" s="1">
+        <v>0.3369973654301071</v>
+      </c>
+    </row>
+    <row r="564" spans="1:8">
+      <c r="A564" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B564" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C564" s="1">
+        <v>0.4219396208815869</v>
+      </c>
+      <c r="D564" s="1">
+        <v>0.137693573417812</v>
+      </c>
+      <c r="E564" s="1">
+        <v>3.064337793030252</v>
+      </c>
+      <c r="F564" s="1">
+        <v>0.002181524385068261</v>
+      </c>
+      <c r="G564" s="1">
+        <v>0.1520651760800537</v>
+      </c>
+      <c r="H564" s="1">
+        <v>0.6918140656831202</v>
+      </c>
+    </row>
+    <row r="565" spans="1:8">
+      <c r="A565" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B565" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C565" s="1">
+        <v>-0.5644110210722605</v>
+      </c>
+      <c r="D565" s="1">
+        <v>0.3782105996043711</v>
+      </c>
+      <c r="E565" s="1">
+        <v>-1.492319415856312</v>
+      </c>
+      <c r="F565" s="1">
+        <v>0.1356154291607063</v>
+      </c>
+      <c r="G565" s="1">
+        <v>-1.305690174868127</v>
+      </c>
+      <c r="H565" s="1">
+        <v>0.1768681327236057</v>
+      </c>
+    </row>
+    <row r="566" spans="1:8">
+      <c r="A566" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B566" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C566" s="1">
+        <v>0.06083883373787775</v>
+      </c>
+      <c r="D566" s="1">
+        <v>0.1539556572827789</v>
+      </c>
+      <c r="E566" s="1">
+        <v>0.3951711474046822</v>
+      </c>
+      <c r="F566" s="1">
+        <v>0.6927165844976992</v>
+      </c>
+      <c r="G566" s="1">
+        <v>-0.2409087097525606</v>
+      </c>
+      <c r="H566" s="1">
+        <v>0.3625863772283161</v>
+      </c>
+    </row>
+    <row r="567" spans="1:8">
+      <c r="A567" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B567" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C567" s="1">
+        <v>-0.04854675083489295</v>
+      </c>
+      <c r="D567" s="1">
+        <v>0.1803060764910035</v>
+      </c>
+      <c r="E567" s="1">
+        <v>-0.2692463381139306</v>
+      </c>
+      <c r="F567" s="1">
+        <v>0.7877401237191684</v>
+      </c>
+      <c r="G567" s="1">
+        <v>-0.4019401669509839</v>
+      </c>
+      <c r="H567" s="1">
+        <v>0.304846665281198</v>
+      </c>
+    </row>
+    <row r="569" spans="1:8">
+      <c r="A569" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="570" spans="1:8">
+      <c r="B570" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C570" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D570" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E570" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F570" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G570" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H570" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="571" spans="1:8">
+      <c r="A571" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B571" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C571" s="1">
+        <v>-3.220011683599902</v>
+      </c>
+      <c r="D571" s="1">
+        <v>0.334120011020034</v>
+      </c>
+      <c r="E571" s="1">
+        <v>-9.637290726076353</v>
+      </c>
+      <c r="F571" s="1">
+        <v>5.563698113841918E-22</v>
+      </c>
+      <c r="G571" s="1">
+        <v>-3.874874871713295</v>
+      </c>
+      <c r="H571" s="1">
+        <v>-2.56514849548651</v>
+      </c>
+    </row>
+    <row r="572" spans="1:8">
+      <c r="A572" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B572" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C572" s="1">
+        <v>-0.6210889478804754</v>
+      </c>
+      <c r="D572" s="1">
+        <v>0.3445620725585516</v>
+      </c>
+      <c r="E572" s="1">
+        <v>-1.802545890406825</v>
+      </c>
+      <c r="F572" s="1">
+        <v>0.07145956144800504</v>
+      </c>
+      <c r="G572" s="1">
+        <v>-1.296418200533713</v>
+      </c>
+      <c r="H572" s="1">
+        <v>0.05424030477276254</v>
+      </c>
+    </row>
+    <row r="573" spans="1:8">
+      <c r="A573" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B573" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C573" s="1">
+        <v>-0.8570839528149715</v>
+      </c>
+      <c r="D573" s="1">
+        <v>0.3362116975673475</v>
+      </c>
+      <c r="E573" s="1">
+        <v>-2.549238943845155</v>
+      </c>
+      <c r="F573" s="1">
+        <v>0.01079583038040089</v>
+      </c>
+      <c r="G573" s="1">
+        <v>-1.516046771228045</v>
+      </c>
+      <c r="H573" s="1">
+        <v>-0.1981211344018976</v>
+      </c>
+    </row>
+    <row r="574" spans="1:8">
+      <c r="A574" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B574" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C574" s="1">
+        <v>-0.3302478916274166</v>
+      </c>
+      <c r="D574" s="1">
+        <v>0.5318169749932339</v>
+      </c>
+      <c r="E574" s="1">
+        <v>-0.6209803506772574</v>
+      </c>
+      <c r="F574" s="1">
+        <v>0.5346125517160372</v>
+      </c>
+      <c r="G574" s="1">
+        <v>-1.372590008981194</v>
+      </c>
+      <c r="H574" s="1">
+        <v>0.7120942257263604</v>
+      </c>
+    </row>
+    <row r="575" spans="1:8">
+      <c r="A575" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B575" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C575" s="1">
+        <v>0.0352677992662145</v>
+      </c>
+      <c r="D575" s="1">
+        <v>0.6182661250172221</v>
+      </c>
+      <c r="E575" s="1">
+        <v>0.05704307229388007</v>
+      </c>
+      <c r="F575" s="1">
+        <v>0.9545108842500244</v>
+      </c>
+      <c r="G575" s="1">
+        <v>-1.176511538628679</v>
+      </c>
+      <c r="H575" s="1">
+        <v>1.247047137161108</v>
+      </c>
+    </row>
+    <row r="576" spans="1:8">
+      <c r="A576" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B576" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C576" s="1">
+        <v>-0.1038711015539725</v>
+      </c>
+      <c r="D576" s="1">
+        <v>0.3170212224799095</v>
+      </c>
+      <c r="E576" s="1">
+        <v>-0.3276471547912068</v>
+      </c>
+      <c r="F576" s="1">
+        <v>0.7431784638610279</v>
+      </c>
+      <c r="G576" s="1">
+        <v>-0.725221279949455</v>
+      </c>
+      <c r="H576" s="1">
+        <v>0.51747907684151</v>
+      </c>
+    </row>
+    <row r="577" spans="1:8">
+      <c r="A577" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B577" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C577" s="1">
+        <v>0.7122488802726732</v>
+      </c>
+      <c r="D577" s="1">
+        <v>0.2344532080234607</v>
+      </c>
+      <c r="E577" s="1">
+        <v>3.037914841418598</v>
+      </c>
+      <c r="F577" s="1">
+        <v>0.002382212641185517</v>
+      </c>
+      <c r="G577" s="1">
+        <v>0.2527290364868129</v>
+      </c>
+      <c r="H577" s="1">
+        <v>1.171768724058533</v>
+      </c>
+    </row>
+    <row r="578" spans="1:8">
+      <c r="A578" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B578" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C578" s="1">
+        <v>-0.4000488552381247</v>
+      </c>
+      <c r="D578" s="1">
+        <v>0.2478392100757799</v>
+      </c>
+      <c r="E578" s="1">
+        <v>-1.614146749078989</v>
+      </c>
+      <c r="F578" s="1">
+        <v>0.1064955992418278</v>
+      </c>
+      <c r="G578" s="1">
+        <v>-0.8858047809435099</v>
+      </c>
+      <c r="H578" s="1">
+        <v>0.08570707046726045</v>
+      </c>
+    </row>
+    <row r="579" spans="1:8">
+      <c r="A579" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B579" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C579" s="1">
+        <v>1.242454074241694</v>
+      </c>
+      <c r="D579" s="1">
+        <v>0.2929321910595102</v>
+      </c>
+      <c r="E579" s="1">
+        <v>4.241439186822882</v>
+      </c>
+      <c r="F579" s="1">
+        <v>2.220910688436206E-05</v>
+      </c>
+      <c r="G579" s="1">
+        <v>0.6683175298526481</v>
+      </c>
+      <c r="H579" s="1">
+        <v>1.81659061863074</v>
+      </c>
+    </row>
+    <row r="580" spans="1:8">
+      <c r="A580" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B580" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C580" s="1">
+        <v>-0.3003199431712367</v>
+      </c>
+      <c r="D580" s="1">
+        <v>0.3268526082213848</v>
+      </c>
+      <c r="E580" s="1">
+        <v>-0.9188237622011665</v>
+      </c>
+      <c r="F580" s="1">
+        <v>0.3581877614335142</v>
+      </c>
+      <c r="G580" s="1">
+        <v>-0.9409392835381313</v>
+      </c>
+      <c r="H580" s="1">
+        <v>0.3402993971956579</v>
+      </c>
+    </row>
+    <row r="581" spans="1:8">
+      <c r="A581" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B581" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C581" s="1">
+        <v>0.4607900789240711</v>
+      </c>
+      <c r="D581" s="1">
+        <v>0.8149821623054956</v>
+      </c>
+      <c r="E581" s="1">
+        <v>0.5653989746481644</v>
+      </c>
+      <c r="F581" s="1">
+        <v>0.571802421835031</v>
+      </c>
+      <c r="G581" s="1">
+        <v>-1.136545607237277</v>
+      </c>
+      <c r="H581" s="1">
+        <v>2.058125765085419</v>
+      </c>
+    </row>
+    <row r="582" spans="1:8">
+      <c r="A582" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B582" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C582" s="1">
+        <v>-0.4937137273535617</v>
+      </c>
+      <c r="D582" s="1">
+        <v>0.416020178557125</v>
+      </c>
+      <c r="E582" s="1">
+        <v>-1.18675427972244</v>
+      </c>
+      <c r="F582" s="1">
+        <v>0.2353245577495998</v>
+      </c>
+      <c r="G582" s="1">
+        <v>-1.309098294167449</v>
+      </c>
+      <c r="H582" s="1">
+        <v>0.3216708394603258</v>
+      </c>
+    </row>
+    <row r="583" spans="1:8">
+      <c r="A583" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B583" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C583" s="1">
+        <v>-0.4431338191330692</v>
+      </c>
+      <c r="D583" s="1">
+        <v>0.4207380126862647</v>
+      </c>
+      <c r="E583" s="1">
+        <v>-1.053229814686377</v>
+      </c>
+      <c r="F583" s="1">
+        <v>0.2922356770200806</v>
+      </c>
+      <c r="G583" s="1">
+        <v>-1.267765170925104</v>
+      </c>
+      <c r="H583" s="1">
+        <v>0.381497532658966</v>
+      </c>
+    </row>
+    <row r="585" spans="1:8">
+      <c r="A585" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="586" spans="1:8">
+      <c r="C586" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D586" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E586" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F586" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G586" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="587" spans="1:8">
+      <c r="A587" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B587" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C587" s="1">
+        <v>5.563698113841918E-22</v>
+      </c>
+      <c r="D587" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E587" s="1">
+        <v>0.03995459144446616</v>
+      </c>
+      <c r="F587" s="1">
+        <v>0.0207569349909226</v>
+      </c>
+      <c r="G587" s="1">
+        <v>0.07690776013859134</v>
+      </c>
+    </row>
+    <row r="588" spans="1:8">
+      <c r="A588" s="2"/>
+      <c r="B588" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C588" s="1">
+        <v>0.01079583038040089</v>
+      </c>
+      <c r="D588" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E588" s="1">
+        <v>0.4243978438104394</v>
+      </c>
+      <c r="F588" s="1">
+        <v>0.2195782163473776</v>
+      </c>
+      <c r="G588" s="1">
+        <v>0.8202704841449596</v>
+      </c>
+    </row>
+    <row r="589" spans="1:8">
+      <c r="A589" s="2"/>
+      <c r="B589" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C589" s="1">
+        <v>0.07145956144800504</v>
+      </c>
+      <c r="E589" s="1">
+        <v>0.5373589629730714</v>
+      </c>
+      <c r="F589" s="1">
+        <v>0.2735096975482971</v>
+      </c>
+      <c r="G589" s="1">
+        <v>1.055738270620206</v>
+      </c>
+    </row>
+    <row r="590" spans="1:8">
+      <c r="A590" s="2"/>
+      <c r="B590" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C590" s="1">
+        <v>0.1064955992418278</v>
+      </c>
+      <c r="E590" s="1">
+        <v>0.6702872981901289</v>
+      </c>
+      <c r="F590" s="1">
+        <v>0.4123821623932147</v>
+      </c>
+      <c r="G590" s="1">
+        <v>1.08948713859893</v>
+      </c>
+    </row>
+    <row r="591" spans="1:8">
+      <c r="A591" s="2"/>
+      <c r="B591" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C591" s="1">
+        <v>0.7431784638610279</v>
+      </c>
+      <c r="E591" s="1">
+        <v>0.901341471448728</v>
+      </c>
+      <c r="F591" s="1">
+        <v>0.4842174094957814</v>
+      </c>
+      <c r="G591" s="1">
+        <v>1.677792727443097</v>
+      </c>
+    </row>
+    <row r="592" spans="1:8">
+      <c r="A592" s="2"/>
+      <c r="B592" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C592" s="1">
+        <v>0.002382212641185517</v>
+      </c>
+      <c r="D592" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E592" s="1">
+        <v>2.038570608738161</v>
+      </c>
+      <c r="F592" s="1">
+        <v>1.287534354732079</v>
+      </c>
+      <c r="G592" s="1">
+        <v>3.227696497213736</v>
+      </c>
+    </row>
+    <row r="593" spans="1:7">
+      <c r="A593" s="2"/>
+      <c r="B593" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C593" s="1">
+        <v>0.2922356770200806</v>
+      </c>
+      <c r="E593" s="1">
+        <v>0.6420212866070356</v>
+      </c>
+      <c r="F593" s="1">
+        <v>0.2814599342758922</v>
+      </c>
+      <c r="G593" s="1">
+        <v>1.464476048845076</v>
+      </c>
+    </row>
+    <row r="594" spans="1:7">
+      <c r="A594" s="2"/>
+      <c r="B594" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C594" s="1">
+        <v>0.2353245577495998</v>
+      </c>
+      <c r="E594" s="1">
+        <v>0.6103554861634233</v>
+      </c>
+      <c r="F594" s="1">
+        <v>0.2700634644280019</v>
+      </c>
+      <c r="G594" s="1">
+        <v>1.379430647084457</v>
+      </c>
+    </row>
+    <row r="595" spans="1:7">
+      <c r="A595" s="2"/>
+      <c r="B595" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C595" s="1">
+        <v>0.3581877614335142</v>
+      </c>
+      <c r="E595" s="1">
+        <v>0.7405812388632619</v>
+      </c>
+      <c r="F595" s="1">
+        <v>0.3902610973256945</v>
+      </c>
+      <c r="G595" s="1">
+        <v>1.405368290907364</v>
+      </c>
+    </row>
+    <row r="596" spans="1:7">
+      <c r="A596" s="2"/>
+      <c r="B596" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C596" s="1">
+        <v>0.571802421835031</v>
+      </c>
+      <c r="E596" s="1">
+        <v>1.585326023003487</v>
+      </c>
+      <c r="F596" s="1">
+        <v>0.3209257127026455</v>
+      </c>
+      <c r="G596" s="1">
+        <v>7.831278391646729</v>
+      </c>
+    </row>
+    <row r="597" spans="1:7">
+      <c r="A597" s="2"/>
+      <c r="B597" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C597" s="1">
+        <v>2.220910688436206E-05</v>
+      </c>
+      <c r="D597" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E597" s="1">
+        <v>3.464104210955284</v>
+      </c>
+      <c r="F597" s="1">
+        <v>1.950952139068036</v>
+      </c>
+      <c r="G597" s="1">
+        <v>6.150852060415233</v>
+      </c>
+    </row>
+    <row r="598" spans="1:7">
+      <c r="A598" s="2"/>
+      <c r="B598" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C598" s="1">
+        <v>0.9545108842500244</v>
+      </c>
+      <c r="E598" s="1">
+        <v>1.035897084136515</v>
+      </c>
+      <c r="F598" s="1">
+        <v>0.3083525404802004</v>
+      </c>
+      <c r="G598" s="1">
+        <v>3.480051655327413</v>
+      </c>
+    </row>
+    <row r="599" spans="1:7">
+      <c r="A599" s="2"/>
+      <c r="B599" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C599" s="1">
+        <v>0.5346125517160372</v>
+      </c>
+      <c r="E599" s="1">
+        <v>0.7187455403448569</v>
+      </c>
+      <c r="F599" s="1">
+        <v>0.2534496718033936</v>
+      </c>
+      <c r="G599" s="1">
+        <v>2.038255358903579</v>
+      </c>
+    </row>
+    <row r="600" spans="1:7">
+      <c r="A600" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B600" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C600" s="1">
+        <v>0.03043827325881311</v>
+      </c>
+      <c r="D600" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E600" s="1">
+        <v>1.252312110337718</v>
+      </c>
+      <c r="F600" s="1">
+        <v>1.021472964764968</v>
+      </c>
+      <c r="G600" s="1">
+        <v>1.535317796745953</v>
+      </c>
+    </row>
+    <row r="601" spans="1:7">
+      <c r="A601" s="2"/>
+      <c r="B601" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C601" s="1">
+        <v>0.4128535534896671</v>
+      </c>
+      <c r="E601" s="1">
+        <v>0.9244774254224465</v>
+      </c>
+      <c r="F601" s="1">
+        <v>0.7660734583340914</v>
+      </c>
+      <c r="G601" s="1">
+        <v>1.115635192445201</v>
+      </c>
+    </row>
+    <row r="602" spans="1:7">
+      <c r="A602" s="2"/>
+      <c r="B602" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C602" s="1">
+        <v>0.1006093927893698</v>
+      </c>
+      <c r="E602" s="1">
+        <v>1.18769498451855</v>
+      </c>
+      <c r="F602" s="1">
+        <v>0.9672277208713215</v>
+      </c>
+      <c r="G602" s="1">
+        <v>1.45841495835104</v>
+      </c>
+    </row>
+    <row r="603" spans="1:7">
+      <c r="A603" s="2"/>
+      <c r="B603" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C603" s="1">
+        <v>0.01095642293665167</v>
+      </c>
+      <c r="D603" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E603" s="1">
+        <v>0.7820236474024518</v>
+      </c>
+      <c r="F603" s="1">
+        <v>0.6470777512348328</v>
+      </c>
+      <c r="G603" s="1">
+        <v>0.945112057908928</v>
+      </c>
+    </row>
+    <row r="604" spans="1:7">
+      <c r="A604" s="2"/>
+      <c r="B604" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C604" s="1">
+        <v>0.0003655703611464461</v>
+      </c>
+      <c r="D604" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E604" s="1">
+        <v>0.5911064315491679</v>
+      </c>
+      <c r="F604" s="1">
+        <v>0.4426788014166658</v>
+      </c>
+      <c r="G604" s="1">
+        <v>0.789300983694307</v>
+      </c>
+    </row>
+    <row r="605" spans="1:7">
+      <c r="A605" s="2"/>
+      <c r="B605" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C605" s="1">
+        <v>0.2909840920523293</v>
+      </c>
+      <c r="E605" s="1">
+        <v>0.904107219360633</v>
+      </c>
+      <c r="F605" s="1">
+        <v>0.7498256731993821</v>
+      </c>
+      <c r="G605" s="1">
+        <v>1.090133204711787</v>
+      </c>
+    </row>
+    <row r="606" spans="1:7">
+      <c r="A606" s="2"/>
+      <c r="B606" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C606" s="1">
+        <v>0.004600712496250168</v>
+      </c>
+      <c r="D606" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E606" s="1">
+        <v>0.5978365170354801</v>
+      </c>
+      <c r="F606" s="1">
+        <v>0.4188465394957133</v>
+      </c>
+      <c r="G606" s="1">
+        <v>0.8533161131793756</v>
+      </c>
+    </row>
+    <row r="607" spans="1:7">
+      <c r="A607" s="2"/>
+      <c r="B607" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C607" s="1">
+        <v>0.4492998724301147</v>
+      </c>
+      <c r="E607" s="1">
+        <v>0.9050556454142124</v>
+      </c>
+      <c r="F607" s="1">
+        <v>0.6989410013783011</v>
+      </c>
+      <c r="G607" s="1">
+        <v>1.171952596400602</v>
+      </c>
+    </row>
+    <row r="608" spans="1:7">
+      <c r="A608" s="2"/>
+      <c r="B608" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C608" s="1">
+        <v>0.5564597044586419</v>
+      </c>
+      <c r="E608" s="1">
+        <v>0.9218935648034727</v>
+      </c>
+      <c r="F608" s="1">
+        <v>0.7030300263827154</v>
+      </c>
+      <c r="G608" s="1">
+        <v>1.208892526538252</v>
+      </c>
+    </row>
+    <row r="609" spans="1:7">
+      <c r="A609" s="2"/>
+      <c r="B609" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C609" s="1">
+        <v>0.01241480255182997</v>
+      </c>
+      <c r="D609" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E609" s="1">
+        <v>0.2603569720001682</v>
+      </c>
+      <c r="F609" s="1">
+        <v>0.09065829954651919</v>
+      </c>
+      <c r="G609" s="1">
+        <v>0.7477059817817746</v>
+      </c>
+    </row>
+    <row r="610" spans="1:7">
+      <c r="A610" s="2"/>
+      <c r="B610" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C610" s="1">
+        <v>8.641755080100111E-20</v>
+      </c>
+      <c r="D610" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E610" s="1">
+        <v>0.4153771398150439</v>
+      </c>
+      <c r="F610" s="1">
+        <v>0.3438000387044616</v>
+      </c>
+      <c r="G610" s="1">
+        <v>0.5018561630507677</v>
+      </c>
+    </row>
+    <row r="611" spans="1:7">
+      <c r="A611" s="2"/>
+      <c r="B611" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C611" s="1">
+        <v>0.679041437636994</v>
+      </c>
+      <c r="E611" s="1">
+        <v>0.907090144857518</v>
+      </c>
+      <c r="F611" s="1">
+        <v>0.5715417577746217</v>
+      </c>
+      <c r="G611" s="1">
+        <v>1.439636771425713</v>
+      </c>
+    </row>
+    <row r="612" spans="1:7">
+      <c r="A612" s="2"/>
+      <c r="B612" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C612" s="1">
+        <v>0.1230465751327812</v>
+      </c>
+      <c r="E612" s="1">
+        <v>1.237814906643693</v>
+      </c>
+      <c r="F612" s="1">
+        <v>0.9438301980585345</v>
+      </c>
+      <c r="G612" s="1">
+        <v>1.623370121300475</v>
+      </c>
+    </row>
+    <row r="613" spans="1:7">
+      <c r="A613" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B613" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C613" s="1">
+        <v>2.635115730555844E-22</v>
+      </c>
+      <c r="D613" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E613" s="1">
+        <v>0.2598298490467053</v>
+      </c>
+      <c r="F613" s="1">
+        <v>0.1979654357731759</v>
+      </c>
+      <c r="G613" s="1">
+        <v>0.3410269585291988</v>
+      </c>
+    </row>
+    <row r="614" spans="1:7">
+      <c r="A614" s="2"/>
+      <c r="B614" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C614" s="1">
+        <v>0.007203775417692744</v>
+      </c>
+      <c r="D614" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E614" s="1">
+        <v>1.356040702488492</v>
+      </c>
+      <c r="F614" s="1">
+        <v>1.085924401402571</v>
+      </c>
+      <c r="G614" s="1">
+        <v>1.69334659432134</v>
+      </c>
+    </row>
+    <row r="615" spans="1:7">
+      <c r="A615" s="2"/>
+      <c r="B615" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C615" s="1">
+        <v>0.7529724151289838</v>
+      </c>
+      <c r="E615" s="1">
+        <v>0.9592207167867117</v>
+      </c>
+      <c r="F615" s="1">
+        <v>0.7401412195747047</v>
+      </c>
+      <c r="G615" s="1">
+        <v>1.243147063261141</v>
+      </c>
+    </row>
+    <row r="616" spans="1:7">
+      <c r="A616" s="2"/>
+      <c r="B616" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C616" s="1">
+        <v>0.7307014160917791</v>
+      </c>
+      <c r="E616" s="1">
+        <v>0.9582502835410031</v>
+      </c>
+      <c r="F616" s="1">
+        <v>0.7516455326701644</v>
+      </c>
+      <c r="G616" s="1">
+        <v>1.221644466700176</v>
+      </c>
+    </row>
+    <row r="617" spans="1:7">
+      <c r="A617" s="2"/>
+      <c r="B617" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C617" s="1">
+        <v>5.358685390828512E-07</v>
+      </c>
+      <c r="D617" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E617" s="1">
+        <v>1.928875342590763</v>
+      </c>
+      <c r="F617" s="1">
+        <v>1.491959695653061</v>
+      </c>
+      <c r="G617" s="1">
+        <v>2.493740345731034</v>
+      </c>
+    </row>
+    <row r="618" spans="1:7">
+      <c r="A618" s="2"/>
+      <c r="B618" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C618" s="1">
+        <v>0.6385747782972211</v>
+      </c>
+      <c r="E618" s="1">
+        <v>1.054434664925491</v>
+      </c>
+      <c r="F618" s="1">
+        <v>0.845204177690837</v>
+      </c>
+      <c r="G618" s="1">
+        <v>1.315460207063985</v>
+      </c>
+    </row>
+    <row r="619" spans="1:7">
+      <c r="A619" s="2"/>
+      <c r="B619" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C619" s="1">
+        <v>0.7877401237191684</v>
+      </c>
+      <c r="E619" s="1">
+        <v>0.9526128028209225</v>
+      </c>
+      <c r="F619" s="1">
+        <v>0.6690207740455918</v>
+      </c>
+      <c r="G619" s="1">
+        <v>1.356417001240222</v>
+      </c>
+    </row>
+    <row r="620" spans="1:7">
+      <c r="A620" s="2"/>
+      <c r="B620" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C620" s="1">
+        <v>0.6927165844976992</v>
+      </c>
+      <c r="E620" s="1">
+        <v>1.062727624545608</v>
+      </c>
+      <c r="F620" s="1">
+        <v>0.7859133693395327</v>
+      </c>
+      <c r="G620" s="1">
+        <v>1.437041343273585</v>
+      </c>
+    </row>
+    <row r="621" spans="1:7">
+      <c r="A621" s="2"/>
+      <c r="B621" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C621" s="1">
+        <v>0.002181524385068261</v>
+      </c>
+      <c r="D621" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E621" s="1">
+        <v>1.524916448792745</v>
+      </c>
+      <c r="F621" s="1">
+        <v>1.164236114305562</v>
+      </c>
+      <c r="G621" s="1">
+        <v>1.997335546652153</v>
+      </c>
+    </row>
+    <row r="622" spans="1:7">
+      <c r="A622" s="2"/>
+      <c r="B622" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C622" s="1">
+        <v>0.1356154291607063</v>
+      </c>
+      <c r="E622" s="1">
+        <v>0.5686949975076856</v>
+      </c>
+      <c r="F622" s="1">
+        <v>0.2709854431474749</v>
+      </c>
+      <c r="G622" s="1">
+        <v>1.193473702623425</v>
+      </c>
+    </row>
+    <row r="623" spans="1:7">
+      <c r="A623" s="2"/>
+      <c r="B623" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C623" s="1">
+        <v>0.3240653368093933</v>
+      </c>
+      <c r="E623" s="1">
+        <v>1.119410169033908</v>
+      </c>
+      <c r="F623" s="1">
+        <v>0.8945866223798794</v>
+      </c>
+      <c r="G623" s="1">
+        <v>1.400735373398431</v>
+      </c>
+    </row>
+    <row r="624" spans="1:7">
+      <c r="A624" s="2"/>
+      <c r="B624" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C624" s="1">
+        <v>0.5721652503803307</v>
+      </c>
+      <c r="E624" s="1">
+        <v>0.8387042337796062</v>
+      </c>
+      <c r="F624" s="1">
+        <v>0.4555621443778501</v>
+      </c>
+      <c r="G624" s="1">
+        <v>1.544080868967912</v>
+      </c>
+    </row>
+    <row r="625" spans="1:7">
+      <c r="A625" s="2"/>
+      <c r="B625" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C625" s="1">
+        <v>0.02904355107345591</v>
+      </c>
+      <c r="D625" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E625" s="1">
+        <v>0.6140322625452493</v>
+      </c>
+      <c r="F625" s="1">
+        <v>0.3962904661805755</v>
+      </c>
+      <c r="G625" s="1">
+        <v>0.9514122887696125</v>
+      </c>
+    </row>
+    <row r="626" spans="1:7">
+      <c r="A626" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B626" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C626" s="1">
+        <v>5.75724982403861E-30</v>
+      </c>
+      <c r="D626" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E626" s="1">
+        <v>0.2001249324129587</v>
+      </c>
+      <c r="F626" s="1">
+        <v>0.1516637311617033</v>
+      </c>
+      <c r="G626" s="1">
+        <v>0.2640709698127507</v>
+      </c>
+    </row>
+    <row r="627" spans="1:7">
+      <c r="A627" s="2"/>
+      <c r="B627" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C627" s="1">
+        <v>0.3653235325354613</v>
+      </c>
+      <c r="E627" s="1">
+        <v>1.10245501444012</v>
+      </c>
+      <c r="F627" s="1">
+        <v>0.892579293611852</v>
+      </c>
+      <c r="G627" s="1">
+        <v>1.361679648590076</v>
+      </c>
+    </row>
+    <row r="628" spans="1:7">
+      <c r="A628" s="2"/>
+      <c r="B628" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C628" s="1">
+        <v>0.19828416430527</v>
+      </c>
+      <c r="E628" s="1">
+        <v>1.166756205614445</v>
+      </c>
+      <c r="F628" s="1">
+        <v>0.9224298515240792</v>
+      </c>
+      <c r="G628" s="1">
+        <v>1.475797906031103</v>
+      </c>
+    </row>
+    <row r="629" spans="1:7">
+      <c r="A629" s="2"/>
+      <c r="B629" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C629" s="1">
+        <v>0.4620668891808699</v>
+      </c>
+      <c r="E629" s="1">
+        <v>1.092949910686558</v>
+      </c>
+      <c r="F629" s="1">
+        <v>0.8624437594233449</v>
+      </c>
+      <c r="G629" s="1">
+        <v>1.385063656867851</v>
+      </c>
+    </row>
+    <row r="630" spans="1:7">
+      <c r="A630" s="2"/>
+      <c r="B630" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C630" s="1">
+        <v>0.2455031605052839</v>
+      </c>
+      <c r="E630" s="1">
+        <v>1.170424426516768</v>
+      </c>
+      <c r="F630" s="1">
+        <v>0.8974331742100226</v>
+      </c>
+      <c r="G630" s="1">
+        <v>1.526457208797716</v>
+      </c>
+    </row>
+    <row r="631" spans="1:7">
+      <c r="A631" s="2"/>
+      <c r="B631" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C631" s="1">
+        <v>0.9489615315521314</v>
+      </c>
+      <c r="E631" s="1">
+        <v>1.006724827909416</v>
+      </c>
+      <c r="F631" s="1">
+        <v>0.8199455391426391</v>
+      </c>
+      <c r="G631" s="1">
+        <v>1.236051457989496</v>
+      </c>
+    </row>
+    <row r="632" spans="1:7">
+      <c r="A632" s="2"/>
+      <c r="B632" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C632" s="1">
+        <v>0.3874835484867725</v>
+      </c>
+      <c r="E632" s="1">
+        <v>1.140395597832054</v>
+      </c>
+      <c r="F632" s="1">
+        <v>0.8465543172678562</v>
+      </c>
+      <c r="G632" s="1">
+        <v>1.536229977246976</v>
+      </c>
+    </row>
+    <row r="633" spans="1:7">
+      <c r="A633" s="2"/>
+      <c r="B633" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C633" s="1">
+        <v>0.3499381433206767</v>
+      </c>
+      <c r="E633" s="1">
+        <v>1.138307054241064</v>
+      </c>
+      <c r="F633" s="1">
+        <v>0.8675424084204794</v>
+      </c>
+      <c r="G633" s="1">
+        <v>1.493578800480897</v>
+      </c>
+    </row>
+    <row r="634" spans="1:7">
+      <c r="A634" s="2"/>
+      <c r="B634" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C634" s="1">
+        <v>0.2610134774064551</v>
+      </c>
+      <c r="E634" s="1">
+        <v>1.161280120378791</v>
+      </c>
+      <c r="F634" s="1">
+        <v>0.8947539858895064</v>
+      </c>
+      <c r="G634" s="1">
+        <v>1.507198111720417</v>
+      </c>
+    </row>
+    <row r="635" spans="1:7">
+      <c r="A635" s="2"/>
+      <c r="B635" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C635" s="1">
+        <v>0.6055075748093981</v>
+      </c>
+      <c r="E635" s="1">
+        <v>1.14514172142013</v>
+      </c>
+      <c r="F635" s="1">
+        <v>0.6847065431039845</v>
+      </c>
+      <c r="G635" s="1">
+        <v>1.915199402348792</v>
+      </c>
+    </row>
+    <row r="636" spans="1:7">
+      <c r="A636" s="2"/>
+      <c r="B636" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C636" s="1">
+        <v>8.503220591470087E-12</v>
+      </c>
+      <c r="D636" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E636" s="1">
+        <v>2.173111801264366</v>
+      </c>
+      <c r="F636" s="1">
+        <v>1.73919727562023</v>
+      </c>
+      <c r="G636" s="1">
+        <v>2.715284210130997</v>
+      </c>
+    </row>
+    <row r="637" spans="1:7">
+      <c r="A637" s="2"/>
+      <c r="B637" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C637" s="1">
+        <v>0.2675161165776037</v>
+      </c>
+      <c r="E637" s="1">
+        <v>1.333233760754325</v>
+      </c>
+      <c r="F637" s="1">
+        <v>0.801893242785563</v>
+      </c>
+      <c r="G637" s="1">
+        <v>2.216644518216063</v>
+      </c>
+    </row>
+    <row r="638" spans="1:7">
+      <c r="A638" s="2"/>
+      <c r="B638" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C638" s="1">
+        <v>0.5892118038207506</v>
+      </c>
+      <c r="E638" s="1">
+        <v>1.105198791434022</v>
+      </c>
+      <c r="F638" s="1">
+        <v>0.7687134442276027</v>
+      </c>
+      <c r="G638" s="1">
+        <v>1.588972298792745</v>
+      </c>
+    </row>
+    <row r="639" spans="1:7">
+      <c r="A639" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B639" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C639" s="1">
+        <v>6.303753463585649E-35</v>
+      </c>
+      <c r="D639" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E639" s="1">
+        <v>0.2091878438075394</v>
+      </c>
+      <c r="F639" s="1">
+        <v>0.1631259205336</v>
+      </c>
+      <c r="G639" s="1">
+        <v>0.2682562884776737</v>
+      </c>
+    </row>
+    <row r="640" spans="1:7">
+      <c r="A640" s="2"/>
+      <c r="B640" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C640" s="1">
+        <v>0.0001144842107323911</v>
+      </c>
+      <c r="D640" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E640" s="1">
+        <v>1.421955873054784</v>
+      </c>
+      <c r="F640" s="1">
+        <v>1.189074004475948</v>
+      </c>
+      <c r="G640" s="1">
+        <v>1.700447993399802</v>
+      </c>
+    </row>
+    <row r="641" spans="1:7">
+      <c r="A641" s="2"/>
+      <c r="B641" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C641" s="1">
+        <v>0.01228218742131392</v>
+      </c>
+      <c r="D641" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E641" s="1">
+        <v>0.7594346512287379</v>
+      </c>
+      <c r="F641" s="1">
+        <v>0.6122710373493028</v>
+      </c>
+      <c r="G641" s="1">
+        <v>0.9419700660410008</v>
+      </c>
+    </row>
+    <row r="642" spans="1:7">
+      <c r="A642" s="2"/>
+      <c r="B642" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C642" s="1">
+        <v>0.4531864316378061</v>
+      </c>
+      <c r="E642" s="1">
+        <v>1.08104171817588</v>
+      </c>
+      <c r="F642" s="1">
+        <v>0.8818928708240604</v>
+      </c>
+      <c r="G642" s="1">
+        <v>1.325162312906154</v>
+      </c>
+    </row>
+    <row r="643" spans="1:7">
+      <c r="A643" s="2"/>
+      <c r="B643" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C643" s="1">
+        <v>1.699538476781488E-08</v>
+      </c>
+      <c r="D643" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E643" s="1">
+        <v>1.821996185558173</v>
+      </c>
+      <c r="F643" s="1">
+        <v>1.479128244363792</v>
+      </c>
+      <c r="G643" s="1">
+        <v>2.244342309626032</v>
+      </c>
+    </row>
+    <row r="644" spans="1:7">
+      <c r="A644" s="2"/>
+      <c r="B644" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C644" s="1">
+        <v>0.0491657849146158</v>
+      </c>
+      <c r="D644" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E644" s="1">
+        <v>1.190649738289375</v>
+      </c>
+      <c r="F644" s="1">
+        <v>1.000637754036729</v>
+      </c>
+      <c r="G644" s="1">
+        <v>1.416743265551941</v>
+      </c>
+    </row>
+    <row r="645" spans="1:7">
+      <c r="A645" s="2"/>
+      <c r="B645" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C645" s="1">
+        <v>0.83055921949477</v>
+      </c>
+      <c r="E645" s="1">
+        <v>0.9714315849866472</v>
+      </c>
+      <c r="F645" s="1">
+        <v>0.7449308970368412</v>
+      </c>
+      <c r="G645" s="1">
+        <v>1.266801159763143</v>
+      </c>
+    </row>
+    <row r="646" spans="1:7">
+      <c r="A646" s="2"/>
+      <c r="B646" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C646" s="1">
+        <v>0.8896330971005005</v>
+      </c>
+      <c r="E646" s="1">
+        <v>0.9829024980175183</v>
+      </c>
+      <c r="F646" s="1">
+        <v>0.7704207850540145</v>
+      </c>
+      <c r="G646" s="1">
+        <v>1.253986573767405</v>
+      </c>
+    </row>
+    <row r="647" spans="1:7">
+      <c r="A647" s="2"/>
+      <c r="B647" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C647" s="1">
+        <v>3.756796141150703E-12</v>
+      </c>
+      <c r="D647" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E647" s="1">
+        <v>2.066407714590961</v>
+      </c>
+      <c r="F647" s="1">
+        <v>1.683726433595495</v>
+      </c>
+      <c r="G647" s="1">
+        <v>2.536065691979798</v>
+      </c>
+    </row>
+    <row r="648" spans="1:7">
+      <c r="A648" s="2"/>
+      <c r="B648" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C648" s="1">
+        <v>0.1367390703151118</v>
+      </c>
+      <c r="E648" s="1">
+        <v>1.415691434320921</v>
+      </c>
+      <c r="F648" s="1">
+        <v>0.8956158168656608</v>
+      </c>
+      <c r="G648" s="1">
+        <v>2.237770034280498</v>
+      </c>
+    </row>
+    <row r="649" spans="1:7">
+      <c r="A649" s="2"/>
+      <c r="B649" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C649" s="1">
+        <v>9.778824029820875E-34</v>
+      </c>
+      <c r="D649" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E649" s="1">
+        <v>3.534043423377875</v>
+      </c>
+      <c r="F649" s="1">
+        <v>2.880771849864578</v>
+      </c>
+      <c r="G649" s="1">
+        <v>4.335457151494842</v>
+      </c>
+    </row>
+    <row r="650" spans="1:7">
+      <c r="A650" s="2"/>
+      <c r="B650" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C650" s="1">
+        <v>0.2292481125687863</v>
+      </c>
+      <c r="E650" s="1">
+        <v>0.7257253052634283</v>
+      </c>
+      <c r="F650" s="1">
+        <v>0.4303341168085028</v>
+      </c>
+      <c r="G650" s="1">
+        <v>1.223879767204388</v>
+      </c>
+    </row>
+    <row r="651" spans="1:7">
+      <c r="A651" s="2"/>
+      <c r="B651" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C651" s="1">
+        <v>0.002412912081644074</v>
+      </c>
+      <c r="D651" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E651" s="1">
+        <v>0.5405982943304075</v>
+      </c>
+      <c r="F651" s="1">
+        <v>0.3633413146542173</v>
+      </c>
+      <c r="G651" s="1">
+        <v>0.8043305400352543</v>
+      </c>
+    </row>
+    <row r="652" spans="1:7">
+      <c r="A652" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B652" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C652" s="1">
+        <v>1.076401634377507E-22</v>
+      </c>
+      <c r="D652" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E652" s="1">
+        <v>0.2764187654845626</v>
+      </c>
+      <c r="F652" s="1">
+        <v>0.2137640919049212</v>
+      </c>
+      <c r="G652" s="1">
+        <v>0.3574376464780358</v>
+      </c>
+    </row>
+    <row r="653" spans="1:7">
+      <c r="A653" s="2"/>
+      <c r="B653" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C653" s="1">
+        <v>0.09047053184849052</v>
+      </c>
+      <c r="E653" s="1">
+        <v>1.195430162828195</v>
+      </c>
+      <c r="F653" s="1">
+        <v>0.972234995414249</v>
+      </c>
+      <c r="G653" s="1">
+        <v>1.469864056467701</v>
+      </c>
+    </row>
+    <row r="654" spans="1:7">
+      <c r="A654" s="2"/>
+      <c r="B654" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C654" s="1">
+        <v>0.09456680576091746</v>
+      </c>
+      <c r="E654" s="1">
+        <v>0.8088436612379578</v>
+      </c>
+      <c r="F654" s="1">
+        <v>0.6307351386972072</v>
+      </c>
+      <c r="G654" s="1">
+        <v>1.037246901569717</v>
+      </c>
+    </row>
+    <row r="655" spans="1:7">
+      <c r="A655" s="2"/>
+      <c r="B655" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C655" s="1">
+        <v>0.2103323207642823</v>
+      </c>
+      <c r="E655" s="1">
+        <v>0.8667356489483163</v>
+      </c>
+      <c r="F655" s="1">
+        <v>0.6929484593430764</v>
+      </c>
+      <c r="G655" s="1">
+        <v>1.084107591306336</v>
+      </c>
+    </row>
+    <row r="656" spans="1:7">
+      <c r="A656" s="2"/>
+      <c r="B656" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C656" s="1">
+        <v>6.908059231390752E-07</v>
+      </c>
+      <c r="D656" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E656" s="1">
+        <v>1.822855450157607</v>
+      </c>
+      <c r="F656" s="1">
+        <v>1.438124639668288</v>
+      </c>
+      <c r="G656" s="1">
+        <v>2.310510438744527</v>
+      </c>
+    </row>
+    <row r="657" spans="1:7">
+      <c r="A657" s="2"/>
+      <c r="B657" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C657" s="1">
+        <v>0.131314363173481</v>
+      </c>
+      <c r="E657" s="1">
+        <v>0.8538203934418375</v>
+      </c>
+      <c r="F657" s="1">
+        <v>0.6953738609813233</v>
+      </c>
+      <c r="G657" s="1">
+        <v>1.048370243926604</v>
+      </c>
+    </row>
+    <row r="658" spans="1:7">
+      <c r="A658" s="2"/>
+      <c r="B658" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C658" s="1">
+        <v>0.04545464566362853</v>
+      </c>
+      <c r="D658" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E658" s="1">
+        <v>0.7061445516222113</v>
+      </c>
+      <c r="F658" s="1">
+        <v>0.5021614388253089</v>
+      </c>
+      <c r="G658" s="1">
+        <v>0.9929876912735229</v>
+      </c>
+    </row>
+    <row r="659" spans="1:7">
+      <c r="A659" s="2"/>
+      <c r="B659" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C659" s="1">
+        <v>0.03817110476886406</v>
+      </c>
+      <c r="D659" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E659" s="1">
+        <v>1.338121078312889</v>
+      </c>
+      <c r="F659" s="1">
+        <v>1.016010597434499</v>
+      </c>
+      <c r="G659" s="1">
+        <v>1.762351716356664</v>
+      </c>
+    </row>
+    <row r="660" spans="1:7">
+      <c r="A660" s="2"/>
+      <c r="B660" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C660" s="1">
+        <v>1.496602319378977E-18</v>
+      </c>
+      <c r="D660" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E660" s="1">
+        <v>2.782400518402144</v>
+      </c>
+      <c r="F660" s="1">
+        <v>2.214744500067124</v>
+      </c>
+      <c r="G660" s="1">
+        <v>3.495551132227617</v>
+      </c>
+    </row>
+    <row r="661" spans="1:7">
+      <c r="A661" s="2"/>
+      <c r="B661" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C661" s="1">
+        <v>0.6485753473899263</v>
+      </c>
+      <c r="E661" s="1">
+        <v>0.8707508811625326</v>
+      </c>
+      <c r="F661" s="1">
+        <v>0.480177567563645</v>
+      </c>
+      <c r="G661" s="1">
+        <v>1.579013990371032</v>
+      </c>
+    </row>
+    <row r="662" spans="1:7">
+      <c r="A662" s="2"/>
+      <c r="B662" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C662" s="1">
+        <v>1.341907416072246E-06</v>
+      </c>
+      <c r="D662" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E662" s="1">
+        <v>1.704436199208412</v>
+      </c>
+      <c r="F662" s="1">
+        <v>1.373012992853989</v>
+      </c>
+      <c r="G662" s="1">
+        <v>2.115859625722389</v>
+      </c>
+    </row>
+    <row r="663" spans="1:7">
+      <c r="A663" s="2"/>
+      <c r="B663" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C663" s="1">
+        <v>0.4662063620866697</v>
+      </c>
+      <c r="E663" s="1">
+        <v>1.20751967892552</v>
+      </c>
+      <c r="F663" s="1">
+        <v>0.7271352108810394</v>
+      </c>
+      <c r="G663" s="1">
+        <v>2.005271857521062</v>
+      </c>
+    </row>
+    <row r="664" spans="1:7">
+      <c r="A664" s="2"/>
+      <c r="B664" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C664" s="1">
+        <v>0.002192984741371619</v>
+      </c>
+      <c r="D664" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E664" s="1">
+        <v>0.4884737595781748</v>
+      </c>
+      <c r="F664" s="1">
+        <v>0.3088309745169134</v>
+      </c>
+      <c r="G664" s="1">
+        <v>0.7726123138058778</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="18">
     <mergeCell ref="A56:A66"/>
     <mergeCell ref="A67:A77"/>
     <mergeCell ref="A78:A88"/>
@@ -10250,6 +14195,12 @@
     <mergeCell ref="A429:A444"/>
     <mergeCell ref="A445:A460"/>
     <mergeCell ref="A461:A476"/>
+    <mergeCell ref="A587:A599"/>
+    <mergeCell ref="A600:A612"/>
+    <mergeCell ref="A613:A625"/>
+    <mergeCell ref="A626:A638"/>
+    <mergeCell ref="A639:A651"/>
+    <mergeCell ref="A652:A664"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added percentage difference for odds ratios
</commit_message>
<xml_diff>
--- a/assets_output/09_logistic_regression_blocks.xlsx
+++ b/assets_output/09_logistic_regression_blocks.xlsx
@@ -49,7 +49,7 @@
     <t>rt_outcome</t>
   </si>
   <si>
-    <t>2026-06-21 13:14</t>
+    <t>2026-06-21 14:26</t>
   </si>
   <si>
     <t>2679</t>
@@ -208,7 +208,7 @@
     <t>cli_outcome</t>
   </si>
   <si>
-    <t>2026-06-21 13:15</t>
+    <t>2026-06-21 14:27</t>
   </si>
   <si>
     <t>2014</t>
@@ -496,7 +496,7 @@
     <t>MNLogit: 'Outcomes from individual placements (vs. forwards moves)', table 0</t>
   </si>
   <si>
-    <t>2026-06-21 13:16</t>
+    <t>2026-06-21 14:28</t>
   </si>
   <si>
     <t>5191</t>
@@ -912,10 +912,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H664"/>
+  <dimension ref="A1:J664"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="8" width="9.140625" style="1"/>
+    <col min="2" max="10" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">

</xml_diff>